<commit_message>
changed R_0805_PTC-Fuse (R170A-H) to 28044 out of TE.DbLib/ FUSE, 62R R_0603 resistors to 23134 out of TE.DbLib/R_1005_0402
</commit_message>
<xml_diff>
--- a/Using Trenz Library/BOM_MissingComponents_in_process_Simon.xlsx
+++ b/Using Trenz Library/BOM_MissingComponents_in_process_Simon.xlsx
@@ -1177,7 +1177,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1214,6 +1214,9 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Link" xfId="1" builtinId="8"/>
@@ -1676,6 +1679,8 @@
       <c r="Q3" s="14" t="s">
         <v>321</v>
       </c>
+      <c r="R3" s="16"/>
+      <c r="S3" s="15"/>
     </row>
     <row r="4" spans="1:19" ht="45" x14ac:dyDescent="0.25">
       <c r="A4" s="12">
@@ -1729,6 +1734,8 @@
       <c r="Q4" s="14" t="s">
         <v>322</v>
       </c>
+      <c r="R4" s="16"/>
+      <c r="S4" s="15"/>
     </row>
     <row r="5" spans="1:19" ht="45" x14ac:dyDescent="0.25">
       <c r="A5" s="3">
@@ -1939,6 +1946,8 @@
       <c r="Q8" s="15" t="s">
         <v>351</v>
       </c>
+      <c r="R8" s="16"/>
+      <c r="S8" s="15"/>
     </row>
     <row r="9" spans="1:19" ht="45" x14ac:dyDescent="0.25">
       <c r="A9" s="3">
@@ -1997,7 +2006,7 @@
       </c>
     </row>
     <row r="10" spans="1:19" ht="45" x14ac:dyDescent="0.25">
-      <c r="A10" s="3">
+      <c r="A10" s="12">
         <v>8</v>
       </c>
       <c r="B10" s="13" t="s">
@@ -2040,6 +2049,8 @@
       <c r="Q10" s="14" t="s">
         <v>330</v>
       </c>
+      <c r="R10" s="16"/>
+      <c r="S10" s="15"/>
     </row>
     <row r="11" spans="1:19" ht="45" x14ac:dyDescent="0.25">
       <c r="A11" s="3">
@@ -2187,49 +2198,51 @@
       </c>
     </row>
     <row r="14" spans="1:19" ht="60" x14ac:dyDescent="0.25">
-      <c r="A14" s="3">
+      <c r="A14" s="12">
         <v>8</v>
       </c>
-      <c r="B14" s="4" t="s">
+      <c r="B14" s="13" t="s">
         <v>282</v>
       </c>
-      <c r="C14" s="4" t="s">
+      <c r="C14" s="13" t="s">
         <v>283</v>
       </c>
-      <c r="D14" s="4" t="s">
+      <c r="D14" s="13" t="s">
         <v>284</v>
       </c>
-      <c r="E14" s="4" t="s">
+      <c r="E14" s="13" t="s">
         <v>285</v>
       </c>
-      <c r="F14" s="4" t="s">
+      <c r="F14" s="13" t="s">
         <v>282</v>
       </c>
-      <c r="G14" s="4" t="s">
+      <c r="G14" s="13" t="s">
         <v>286</v>
       </c>
-      <c r="H14" s="4" t="s">
+      <c r="H14" s="13" t="s">
         <v>287</v>
       </c>
-      <c r="I14" s="4" t="s">
+      <c r="I14" s="13" t="s">
         <v>288</v>
       </c>
-      <c r="J14" s="4" t="s">
+      <c r="J14" s="13" t="s">
         <v>25</v>
       </c>
-      <c r="K14" s="4" t="s">
+      <c r="K14" s="13" t="s">
         <v>289</v>
       </c>
-      <c r="L14" s="3"/>
-      <c r="M14" s="3"/>
-      <c r="N14" s="3"/>
-      <c r="O14" s="3"/>
-      <c r="P14" s="4" t="s">
-        <v>47</v>
-      </c>
-      <c r="Q14" s="10" t="s">
+      <c r="L14" s="12"/>
+      <c r="M14" s="12"/>
+      <c r="N14" s="12"/>
+      <c r="O14" s="12"/>
+      <c r="P14" s="13" t="s">
+        <v>47</v>
+      </c>
+      <c r="Q14" s="14" t="s">
         <v>333</v>
       </c>
+      <c r="R14" s="16"/>
+      <c r="S14" s="15"/>
     </row>
     <row r="15" spans="1:19" ht="45" x14ac:dyDescent="0.25">
       <c r="A15" s="3">
@@ -2373,49 +2386,51 @@
       </c>
     </row>
     <row r="18" spans="1:20" ht="90" x14ac:dyDescent="0.25">
-      <c r="A18" s="3">
+      <c r="A18" s="12">
         <v>12</v>
       </c>
-      <c r="B18" s="4" t="s">
+      <c r="B18" s="13" t="s">
         <v>308</v>
       </c>
-      <c r="C18" s="4" t="s">
+      <c r="C18" s="13" t="s">
         <v>309</v>
       </c>
-      <c r="D18" s="4" t="s">
+      <c r="D18" s="13" t="s">
         <v>41</v>
       </c>
-      <c r="E18" s="4" t="s">
+      <c r="E18" s="13" t="s">
         <v>310</v>
       </c>
-      <c r="F18" s="4" t="s">
+      <c r="F18" s="13" t="s">
         <v>308</v>
       </c>
-      <c r="G18" s="4" t="s">
+      <c r="G18" s="13" t="s">
         <v>52</v>
       </c>
-      <c r="H18" s="4" t="s">
+      <c r="H18" s="13" t="s">
         <v>53</v>
       </c>
-      <c r="I18" s="4" t="s">
+      <c r="I18" s="13" t="s">
         <v>54</v>
       </c>
-      <c r="J18" s="4" t="s">
+      <c r="J18" s="13" t="s">
         <v>23</v>
       </c>
-      <c r="K18" s="4" t="s">
+      <c r="K18" s="13" t="s">
         <v>311</v>
       </c>
-      <c r="L18" s="3"/>
-      <c r="M18" s="3"/>
-      <c r="N18" s="3"/>
-      <c r="O18" s="3"/>
-      <c r="P18" s="4" t="s">
-        <v>47</v>
-      </c>
-      <c r="Q18" t="s">
+      <c r="L18" s="12"/>
+      <c r="M18" s="12"/>
+      <c r="N18" s="12"/>
+      <c r="O18" s="12"/>
+      <c r="P18" s="13" t="s">
+        <v>47</v>
+      </c>
+      <c r="Q18" s="15" t="s">
         <v>340</v>
       </c>
+      <c r="R18" s="16"/>
+      <c r="S18" s="15"/>
     </row>
     <row r="19" spans="1:20" ht="30" x14ac:dyDescent="0.25">
       <c r="A19" s="3">

</xml_diff>

<commit_message>
changed ESDCAN01-BLY (D5) to 27400 out of TE.DbLib/DIODE, ATP108-TL-H ONSC_PMOS_ATP108 (T8,T11) to 27247 out of TE.DbLib/TRANSISTOR
</commit_message>
<xml_diff>
--- a/Using Trenz Library/BOM_MissingComponents_in_process_Simon.xlsx
+++ b/Using Trenz Library/BOM_MissingComponents_in_process_Simon.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="635" uniqueCount="353">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="635" uniqueCount="354">
   <si>
     <t>Quantity</t>
   </si>
@@ -1086,13 +1086,28 @@
   </si>
   <si>
     <t>CDSOT23-T24CAN</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">double-check </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>discuss</t>
+    </r>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1104,6 +1119,13 @@
       <u/>
       <sz val="11"/>
       <color theme="10"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -1129,7 +1151,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="4">
+  <borders count="5">
     <border>
       <left/>
       <right/>
@@ -1172,12 +1194,27 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color rgb="FFFF0000"/>
+      </left>
+      <right style="medium">
+        <color rgb="FFFF0000"/>
+      </right>
+      <top style="medium">
+        <color rgb="FFFF0000"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FFFF0000"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1215,6 +1252,9 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1950,55 +1990,55 @@
       <c r="S8" s="15"/>
     </row>
     <row r="9" spans="1:19" ht="45" x14ac:dyDescent="0.25">
-      <c r="A9" s="3">
+      <c r="A9" s="12">
         <v>2</v>
       </c>
-      <c r="B9" s="4" t="s">
+      <c r="B9" s="13" t="s">
         <v>182</v>
       </c>
-      <c r="C9" s="4" t="s">
+      <c r="C9" s="13" t="s">
         <v>183</v>
       </c>
-      <c r="D9" s="4" t="s">
+      <c r="D9" s="13" t="s">
         <v>184</v>
       </c>
-      <c r="E9" s="4" t="s">
+      <c r="E9" s="13" t="s">
         <v>182</v>
       </c>
-      <c r="F9" s="4" t="s">
+      <c r="F9" s="13" t="s">
         <v>182</v>
       </c>
-      <c r="G9" s="4" t="s">
+      <c r="G9" s="13" t="s">
         <v>185</v>
       </c>
-      <c r="H9" s="4" t="s">
+      <c r="H9" s="13" t="s">
         <v>186</v>
       </c>
-      <c r="I9" s="4" t="s">
+      <c r="I9" s="13" t="s">
         <v>186</v>
       </c>
-      <c r="J9" s="4" t="s">
+      <c r="J9" s="13" t="s">
         <v>23</v>
       </c>
-      <c r="K9" s="4" t="s">
+      <c r="K9" s="13" t="s">
         <v>187</v>
       </c>
-      <c r="L9" s="4" t="s">
+      <c r="L9" s="13" t="s">
         <v>25</v>
       </c>
-      <c r="M9" s="4" t="s">
+      <c r="M9" s="13" t="s">
         <v>188</v>
       </c>
-      <c r="N9" s="4" t="s">
+      <c r="N9" s="13" t="s">
         <v>36</v>
       </c>
-      <c r="O9" s="4" t="s">
+      <c r="O9" s="13" t="s">
         <v>189</v>
       </c>
-      <c r="P9" s="4" t="s">
-        <v>47</v>
-      </c>
-      <c r="Q9" t="s">
+      <c r="P9" s="13" t="s">
+        <v>47</v>
+      </c>
+      <c r="Q9" s="15" t="s">
         <v>352</v>
       </c>
       <c r="R9" s="7" t="s">
@@ -2525,7 +2565,7 @@
         <v>335</v>
       </c>
     </row>
-    <row r="21" spans="1:20" ht="45" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:20" ht="45.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A21" s="3">
         <v>9</v>
       </c>
@@ -2570,60 +2610,60 @@
         <v>334</v>
       </c>
     </row>
-    <row r="22" spans="1:20" ht="45" x14ac:dyDescent="0.25">
-      <c r="A22" s="3">
+    <row r="22" spans="1:20" ht="45.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A22" s="12">
         <v>2</v>
       </c>
-      <c r="B22" s="4" t="s">
+      <c r="B22" s="13" t="s">
         <v>174</v>
       </c>
-      <c r="C22" s="4" t="s">
+      <c r="C22" s="13" t="s">
         <v>175</v>
       </c>
-      <c r="D22" s="4" t="s">
+      <c r="D22" s="13" t="s">
         <v>76</v>
       </c>
-      <c r="E22" s="4" t="s">
+      <c r="E22" s="13" t="s">
         <v>174</v>
       </c>
-      <c r="F22" s="4" t="s">
+      <c r="F22" s="13" t="s">
         <v>174</v>
       </c>
-      <c r="G22" s="4" t="s">
+      <c r="G22" s="13" t="s">
         <v>176</v>
       </c>
-      <c r="H22" s="4" t="s">
+      <c r="H22" s="13" t="s">
         <v>177</v>
       </c>
-      <c r="I22" s="4" t="s">
+      <c r="I22" s="13" t="s">
         <v>178</v>
       </c>
-      <c r="J22" s="4" t="s">
+      <c r="J22" s="13" t="s">
         <v>25</v>
       </c>
-      <c r="K22" s="4" t="s">
+      <c r="K22" s="13" t="s">
         <v>179</v>
       </c>
-      <c r="L22" s="4" t="s">
+      <c r="L22" s="13" t="s">
         <v>23</v>
       </c>
-      <c r="M22" s="4" t="s">
+      <c r="M22" s="13" t="s">
         <v>180</v>
       </c>
-      <c r="N22" s="4" t="s">
+      <c r="N22" s="13" t="s">
         <v>36</v>
       </c>
-      <c r="O22" s="4" t="s">
+      <c r="O22" s="13" t="s">
         <v>181</v>
       </c>
-      <c r="P22" s="4" t="s">
-        <v>47</v>
-      </c>
-      <c r="Q22" t="s">
+      <c r="P22" s="13" t="s">
+        <v>47</v>
+      </c>
+      <c r="Q22" s="15" t="s">
         <v>341</v>
       </c>
-      <c r="R22" s="7" t="s">
-        <v>342</v>
+      <c r="R22" s="17" t="s">
+        <v>353</v>
       </c>
     </row>
     <row r="23" spans="1:20" ht="30" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
changed 51R R_0603_Array_4R (EXB-38V5103V) to 22843 out of TE.DbLib/R_NET
</commit_message>
<xml_diff>
--- a/Using Trenz Library/BOM_MissingComponents_in_process_Simon.xlsx
+++ b/Using Trenz Library/BOM_MissingComponents_in_process_Simon.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="635" uniqueCount="354">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="637" uniqueCount="356">
   <si>
     <t>Quantity</t>
   </si>
@@ -1088,26 +1088,20 @@
     <t>CDSOT23-T24CAN</t>
   </si>
   <si>
-    <r>
-      <t xml:space="preserve">double-check </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FFFF0000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>discuss</t>
-    </r>
+    <t>used 22843 4fach</t>
+  </si>
+  <si>
+    <t xml:space="preserve">double-check </t>
+  </si>
+  <si>
+    <t>discuss</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1126,6 +1120,13 @@
     <font>
       <sz val="11"/>
       <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="9"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -1151,7 +1152,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="5">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -1195,16 +1196,27 @@
       <diagonal/>
     </border>
     <border>
-      <left style="medium">
+      <left style="thin">
         <color rgb="FFFF0000"/>
       </left>
-      <right style="medium">
+      <right/>
+      <top style="thin">
+        <color rgb="FFFF0000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFFF0000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
         <color rgb="FFFF0000"/>
       </right>
-      <top style="medium">
+      <top style="thin">
         <color rgb="FFFF0000"/>
       </top>
-      <bottom style="medium">
+      <bottom style="thin">
         <color rgb="FFFF0000"/>
       </bottom>
       <diagonal/>
@@ -1214,7 +1226,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1254,9 +1266,13 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Link" xfId="1" builtinId="8"/>
@@ -2329,7 +2345,7 @@
         <v>334</v>
       </c>
     </row>
-    <row r="16" spans="1:19" ht="30" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:19" ht="45" x14ac:dyDescent="0.25">
       <c r="A16" s="3">
         <v>2</v>
       </c>
@@ -2373,56 +2389,59 @@
       <c r="Q16" t="s">
         <v>324</v>
       </c>
-      <c r="R16" t="s">
+      <c r="R16" s="7" t="s">
         <v>335</v>
       </c>
     </row>
     <row r="17" spans="1:20" ht="210" x14ac:dyDescent="0.25">
-      <c r="A17" s="3">
+      <c r="A17" s="12">
         <v>40</v>
       </c>
-      <c r="B17" s="4" t="s">
+      <c r="B17" s="13" t="s">
         <v>312</v>
       </c>
-      <c r="C17" s="4" t="s">
+      <c r="C17" s="13" t="s">
         <v>313</v>
       </c>
-      <c r="D17" s="4" t="s">
+      <c r="D17" s="13" t="s">
         <v>50</v>
       </c>
-      <c r="E17" s="4" t="s">
+      <c r="E17" s="13" t="s">
         <v>314</v>
       </c>
-      <c r="F17" s="4" t="s">
+      <c r="F17" s="13" t="s">
         <v>312</v>
       </c>
-      <c r="G17" s="4" t="s">
+      <c r="G17" s="13" t="s">
         <v>315</v>
       </c>
-      <c r="H17" s="4" t="s">
+      <c r="H17" s="13" t="s">
         <v>316</v>
       </c>
-      <c r="I17" s="4" t="s">
+      <c r="I17" s="13" t="s">
         <v>317</v>
       </c>
-      <c r="J17" s="4" t="s">
+      <c r="J17" s="13" t="s">
         <v>25</v>
       </c>
-      <c r="K17" s="4" t="s">
+      <c r="K17" s="13" t="s">
         <v>318</v>
       </c>
-      <c r="L17" s="3"/>
-      <c r="M17" s="3"/>
-      <c r="N17" s="3"/>
-      <c r="O17" s="3"/>
-      <c r="P17" s="4" t="s">
-        <v>47</v>
-      </c>
-      <c r="Q17" s="10" t="s">
+      <c r="L17" s="12"/>
+      <c r="M17" s="12"/>
+      <c r="N17" s="12"/>
+      <c r="O17" s="12"/>
+      <c r="P17" s="13" t="s">
+        <v>47</v>
+      </c>
+      <c r="Q17" s="14" t="s">
         <v>337</v>
       </c>
-      <c r="R17" s="7" t="s">
+      <c r="R17" s="16" t="s">
         <v>338</v>
+      </c>
+      <c r="S17" s="17" t="s">
+        <v>353</v>
       </c>
     </row>
     <row r="18" spans="1:20" ht="90" x14ac:dyDescent="0.25">
@@ -2517,7 +2536,7 @@
         <v>335</v>
       </c>
     </row>
-    <row r="20" spans="1:20" ht="30" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:20" ht="45" x14ac:dyDescent="0.25">
       <c r="A20" s="3">
         <v>1</v>
       </c>
@@ -2561,11 +2580,11 @@
       <c r="Q20" t="s">
         <v>336</v>
       </c>
-      <c r="R20" t="s">
+      <c r="R20" s="7" t="s">
         <v>335</v>
       </c>
     </row>
-    <row r="21" spans="1:20" ht="45.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:20" ht="45" x14ac:dyDescent="0.25">
       <c r="A21" s="3">
         <v>9</v>
       </c>
@@ -2610,7 +2629,7 @@
         <v>334</v>
       </c>
     </row>
-    <row r="22" spans="1:20" ht="45.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:20" ht="45" x14ac:dyDescent="0.25">
       <c r="A22" s="12">
         <v>2</v>
       </c>
@@ -2662,8 +2681,11 @@
       <c r="Q22" s="15" t="s">
         <v>341</v>
       </c>
-      <c r="R22" s="17" t="s">
-        <v>353</v>
+      <c r="R22" s="18" t="s">
+        <v>354</v>
+      </c>
+      <c r="S22" s="19" t="s">
+        <v>355</v>
       </c>
     </row>
     <row r="23" spans="1:20" ht="30" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
changed 1k91 R_0603 (R94) to 28021 out of TE.DbLib/R_1005_0402
</commit_message>
<xml_diff>
--- a/Using Trenz Library/BOM_MissingComponents_in_process_Simon.xlsx
+++ b/Using Trenz Library/BOM_MissingComponents_in_process_Simon.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="637" uniqueCount="356">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="638" uniqueCount="357">
   <si>
     <t>Quantity</t>
   </si>
@@ -1095,6 +1095,9 @@
   </si>
   <si>
     <t>discuss</t>
+  </si>
+  <si>
+    <t xml:space="preserve">used 0402 </t>
   </si>
 </sst>
 </file>
@@ -1226,7 +1229,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1273,6 +1276,7 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Link" xfId="1" builtinId="8"/>
@@ -2537,51 +2541,54 @@
       </c>
     </row>
     <row r="20" spans="1:20" ht="45" x14ac:dyDescent="0.25">
-      <c r="A20" s="3">
+      <c r="A20" s="12">
         <v>1</v>
       </c>
-      <c r="B20" s="4" t="s">
+      <c r="B20" s="13" t="s">
         <v>48</v>
       </c>
-      <c r="C20" s="4" t="s">
+      <c r="C20" s="13" t="s">
         <v>49</v>
       </c>
-      <c r="D20" s="4" t="s">
+      <c r="D20" s="13" t="s">
         <v>50</v>
       </c>
-      <c r="E20" s="4" t="s">
+      <c r="E20" s="13" t="s">
         <v>51</v>
       </c>
-      <c r="F20" s="4" t="s">
+      <c r="F20" s="13" t="s">
         <v>48</v>
       </c>
-      <c r="G20" s="4" t="s">
+      <c r="G20" s="13" t="s">
         <v>52</v>
       </c>
-      <c r="H20" s="4" t="s">
+      <c r="H20" s="13" t="s">
         <v>53</v>
       </c>
-      <c r="I20" s="4" t="s">
+      <c r="I20" s="13" t="s">
         <v>54</v>
       </c>
-      <c r="J20" s="4" t="s">
+      <c r="J20" s="13" t="s">
         <v>23</v>
       </c>
-      <c r="K20" s="4" t="s">
+      <c r="K20" s="13" t="s">
         <v>55</v>
       </c>
-      <c r="L20" s="3"/>
-      <c r="M20" s="3"/>
-      <c r="N20" s="3"/>
-      <c r="O20" s="3"/>
-      <c r="P20" s="4" t="s">
-        <v>47</v>
-      </c>
-      <c r="Q20" t="s">
+      <c r="L20" s="12"/>
+      <c r="M20" s="12"/>
+      <c r="N20" s="12"/>
+      <c r="O20" s="12"/>
+      <c r="P20" s="13" t="s">
+        <v>47</v>
+      </c>
+      <c r="Q20" s="15" t="s">
         <v>336</v>
       </c>
-      <c r="R20" s="7" t="s">
+      <c r="R20" s="16" t="s">
         <v>335</v>
+      </c>
+      <c r="S20" s="20" t="s">
+        <v>356</v>
       </c>
     </row>
     <row r="21" spans="1:20" ht="45" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
changed 74AHC1G146W,125 (U5A,U5B) to 25648 out of TE.DbLib/LOGIC, SiT8924,4MHz (U1) to 29707 out of TE.DbLib/CLK
</commit_message>
<xml_diff>
--- a/Using Trenz Library/BOM_MissingComponents_in_process_Simon.xlsx
+++ b/Using Trenz Library/BOM_MissingComponents_in_process_Simon.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="638" uniqueCount="357">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="638" uniqueCount="358">
   <si>
     <t>Quantity</t>
   </si>
@@ -1061,9 +1061,6 @@
     <t xml:space="preserve">non-automotive? </t>
   </si>
   <si>
-    <t>SiT8008BI-73-33S-4.000000E</t>
-  </si>
-  <si>
     <t xml:space="preserve">any or-gate </t>
   </si>
   <si>
@@ -1098,6 +1095,12 @@
   </si>
   <si>
     <t xml:space="preserve">used 0402 </t>
+  </si>
+  <si>
+    <t>double-check            29707 SiT8008BI-73-33S-4.000000E</t>
+  </si>
+  <si>
+    <t>used 29707</t>
   </si>
 </sst>
 </file>
@@ -1229,7 +1232,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1277,6 +1280,9 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Link" xfId="1" builtinId="8"/>
@@ -1561,7 +1567,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:T44"/>
+  <dimension ref="A1:S44"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="9" customWidth="1"/>
@@ -1581,6 +1587,7 @@
     <col min="16" max="16" width="16" customWidth="1"/>
     <col min="17" max="17" width="40.140625" customWidth="1"/>
     <col min="18" max="18" width="24.42578125" style="7" customWidth="1"/>
+    <col min="19" max="19" width="14.140625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:19" s="1" customFormat="1" ht="60" x14ac:dyDescent="0.25">
@@ -1959,7 +1966,7 @@
         <v>47</v>
       </c>
       <c r="Q7" t="s">
-        <v>350</v>
+        <v>349</v>
       </c>
     </row>
     <row r="8" spans="1:19" ht="30" x14ac:dyDescent="0.25">
@@ -2004,7 +2011,7 @@
         <v>47</v>
       </c>
       <c r="Q8" s="15" t="s">
-        <v>351</v>
+        <v>350</v>
       </c>
       <c r="R8" s="16"/>
       <c r="S8" s="15"/>
@@ -2059,7 +2066,7 @@
         <v>47</v>
       </c>
       <c r="Q9" s="15" t="s">
-        <v>352</v>
+        <v>351</v>
       </c>
       <c r="R9" s="7" t="s">
         <v>342</v>
@@ -2397,7 +2404,7 @@
         <v>335</v>
       </c>
     </row>
-    <row r="17" spans="1:20" ht="210" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:19" ht="210" x14ac:dyDescent="0.25">
       <c r="A17" s="12">
         <v>40</v>
       </c>
@@ -2445,10 +2452,10 @@
         <v>338</v>
       </c>
       <c r="S17" s="17" t="s">
-        <v>353</v>
-      </c>
-    </row>
-    <row r="18" spans="1:20" ht="90" x14ac:dyDescent="0.25">
+        <v>352</v>
+      </c>
+    </row>
+    <row r="18" spans="1:19" ht="90" x14ac:dyDescent="0.25">
       <c r="A18" s="12">
         <v>12</v>
       </c>
@@ -2495,7 +2502,7 @@
       <c r="R18" s="16"/>
       <c r="S18" s="15"/>
     </row>
-    <row r="19" spans="1:20" ht="30" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:19" ht="30" x14ac:dyDescent="0.25">
       <c r="A19" s="3">
         <v>4</v>
       </c>
@@ -2540,7 +2547,7 @@
         <v>335</v>
       </c>
     </row>
-    <row r="20" spans="1:20" ht="45" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:19" ht="45" x14ac:dyDescent="0.25">
       <c r="A20" s="12">
         <v>1</v>
       </c>
@@ -2588,10 +2595,10 @@
         <v>335</v>
       </c>
       <c r="S20" s="20" t="s">
-        <v>356</v>
-      </c>
-    </row>
-    <row r="21" spans="1:20" ht="45" x14ac:dyDescent="0.25">
+        <v>355</v>
+      </c>
+    </row>
+    <row r="21" spans="1:19" ht="45" x14ac:dyDescent="0.25">
       <c r="A21" s="3">
         <v>9</v>
       </c>
@@ -2636,7 +2643,7 @@
         <v>334</v>
       </c>
     </row>
-    <row r="22" spans="1:20" ht="45" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:19" ht="45" x14ac:dyDescent="0.25">
       <c r="A22" s="12">
         <v>2</v>
       </c>
@@ -2689,67 +2696,64 @@
         <v>341</v>
       </c>
       <c r="R22" s="18" t="s">
+        <v>353</v>
+      </c>
+      <c r="S22" s="19" t="s">
         <v>354</v>
       </c>
-      <c r="S22" s="19" t="s">
-        <v>355</v>
-      </c>
-    </row>
-    <row r="23" spans="1:20" ht="30" x14ac:dyDescent="0.25">
-      <c r="A23" s="3">
+    </row>
+    <row r="23" spans="1:19" ht="45" x14ac:dyDescent="0.25">
+      <c r="A23" s="12">
         <v>1</v>
       </c>
-      <c r="B23" s="4" t="s">
+      <c r="B23" s="13" t="s">
         <v>126</v>
       </c>
-      <c r="C23" s="4" t="s">
+      <c r="C23" s="13" t="s">
         <v>127</v>
       </c>
-      <c r="D23" s="4" t="s">
+      <c r="D23" s="13" t="s">
         <v>128</v>
       </c>
-      <c r="E23" s="4" t="s">
+      <c r="E23" s="13" t="s">
         <v>129</v>
       </c>
-      <c r="F23" s="4" t="s">
+      <c r="F23" s="13" t="s">
         <v>126</v>
       </c>
-      <c r="G23" s="4" t="s">
+      <c r="G23" s="13" t="s">
         <v>130</v>
       </c>
-      <c r="H23" s="4" t="s">
+      <c r="H23" s="13" t="s">
         <v>131</v>
       </c>
-      <c r="I23" s="4" t="s">
+      <c r="I23" s="13" t="s">
         <v>132</v>
       </c>
-      <c r="J23" s="4" t="s">
+      <c r="J23" s="13" t="s">
         <v>36</v>
       </c>
-      <c r="K23" s="4" t="s">
+      <c r="K23" s="13" t="s">
         <v>133</v>
       </c>
-      <c r="L23" s="3"/>
-      <c r="M23" s="3"/>
-      <c r="N23" s="3"/>
-      <c r="O23" s="3"/>
-      <c r="P23" s="4" t="s">
-        <v>47</v>
-      </c>
-      <c r="Q23" t="s">
+      <c r="L23" s="12"/>
+      <c r="M23" s="12"/>
+      <c r="N23" s="12"/>
+      <c r="O23" s="12"/>
+      <c r="P23" s="13" t="s">
+        <v>47</v>
+      </c>
+      <c r="Q23" s="15" t="s">
         <v>343</v>
       </c>
-      <c r="R23" s="7">
-        <v>29707</v>
-      </c>
-      <c r="S23" t="s">
-        <v>344</v>
-      </c>
-      <c r="T23" t="s">
-        <v>342</v>
-      </c>
-    </row>
-    <row r="24" spans="1:20" ht="45" x14ac:dyDescent="0.25">
+      <c r="R23" s="7" t="s">
+        <v>356</v>
+      </c>
+      <c r="S23" s="20" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="24" spans="1:19" ht="45" x14ac:dyDescent="0.25">
       <c r="A24" s="3">
         <v>3</v>
       </c>
@@ -2798,7 +2802,7 @@
         <v>334</v>
       </c>
     </row>
-    <row r="25" spans="1:20" ht="60" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:19" ht="60" x14ac:dyDescent="0.25">
       <c r="A25" s="3">
         <v>2</v>
       </c>
@@ -2844,10 +2848,10 @@
         <v>38</v>
       </c>
       <c r="Q25" s="5" t="s">
-        <v>345</v>
-      </c>
-    </row>
-    <row r="26" spans="1:20" ht="45" x14ac:dyDescent="0.25">
+        <v>344</v>
+      </c>
+    </row>
+    <row r="26" spans="1:19" ht="45" x14ac:dyDescent="0.25">
       <c r="A26" s="3">
         <v>1</v>
       </c>
@@ -2893,13 +2897,13 @@
         <v>47</v>
       </c>
       <c r="Q26" s="5" t="s">
-        <v>347</v>
+        <v>346</v>
       </c>
       <c r="R26" s="7" t="s">
-        <v>349</v>
-      </c>
-    </row>
-    <row r="27" spans="1:20" ht="90" x14ac:dyDescent="0.25">
+        <v>348</v>
+      </c>
+    </row>
+    <row r="27" spans="1:19" ht="90" x14ac:dyDescent="0.25">
       <c r="A27" s="3">
         <v>1</v>
       </c>
@@ -2949,13 +2953,13 @@
         <v>47</v>
       </c>
       <c r="Q27" s="5" t="s">
-        <v>347</v>
+        <v>346</v>
       </c>
       <c r="R27" s="7" t="s">
-        <v>346</v>
-      </c>
-    </row>
-    <row r="28" spans="1:20" ht="45" x14ac:dyDescent="0.25">
+        <v>345</v>
+      </c>
+    </row>
+    <row r="28" spans="1:19" ht="45" x14ac:dyDescent="0.25">
       <c r="A28" s="3">
         <v>2</v>
       </c>
@@ -2997,13 +3001,13 @@
         <v>47</v>
       </c>
       <c r="Q28" t="s">
-        <v>347</v>
+        <v>346</v>
       </c>
       <c r="R28" s="7" t="s">
-        <v>349</v>
-      </c>
-    </row>
-    <row r="29" spans="1:20" ht="60" x14ac:dyDescent="0.25">
+        <v>348</v>
+      </c>
+    </row>
+    <row r="29" spans="1:19" ht="60" x14ac:dyDescent="0.25">
       <c r="A29" s="3">
         <v>1</v>
       </c>
@@ -3056,7 +3060,7 @@
         <v>323</v>
       </c>
     </row>
-    <row r="30" spans="1:20" ht="45" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:19" ht="45" x14ac:dyDescent="0.25">
       <c r="A30" s="3">
         <v>5</v>
       </c>
@@ -3105,63 +3109,63 @@
         <v>323</v>
       </c>
     </row>
-    <row r="31" spans="1:20" ht="60" x14ac:dyDescent="0.25">
-      <c r="A31" s="3">
+    <row r="31" spans="1:19" ht="60" x14ac:dyDescent="0.25">
+      <c r="A31" s="12">
         <v>5</v>
       </c>
-      <c r="B31" s="4" t="s">
+      <c r="B31" s="13" t="s">
         <v>247</v>
       </c>
-      <c r="C31" s="4" t="s">
+      <c r="C31" s="13" t="s">
         <v>248</v>
       </c>
-      <c r="D31" s="4" t="s">
+      <c r="D31" s="13" t="s">
         <v>249</v>
       </c>
-      <c r="E31" s="4" t="s">
+      <c r="E31" s="13" t="s">
         <v>247</v>
       </c>
-      <c r="F31" s="4" t="s">
+      <c r="F31" s="13" t="s">
         <v>247</v>
       </c>
-      <c r="G31" s="4" t="s">
+      <c r="G31" s="13" t="s">
         <v>250</v>
       </c>
-      <c r="H31" s="4" t="s">
+      <c r="H31" s="13" t="s">
         <v>251</v>
       </c>
-      <c r="I31" s="4" t="s">
+      <c r="I31" s="13" t="s">
         <v>252</v>
       </c>
-      <c r="J31" s="4" t="s">
+      <c r="J31" s="13" t="s">
         <v>36</v>
       </c>
-      <c r="K31" s="4" t="s">
+      <c r="K31" s="13" t="s">
         <v>253</v>
       </c>
-      <c r="L31" s="4" t="s">
+      <c r="L31" s="13" t="s">
         <v>25</v>
       </c>
-      <c r="M31" s="4" t="s">
+      <c r="M31" s="13" t="s">
         <v>254</v>
       </c>
-      <c r="N31" s="4" t="s">
+      <c r="N31" s="13" t="s">
         <v>23</v>
       </c>
-      <c r="O31" s="4" t="s">
+      <c r="O31" s="13" t="s">
         <v>255</v>
       </c>
-      <c r="P31" s="4" t="s">
-        <v>47</v>
-      </c>
-      <c r="Q31" s="10" t="s">
-        <v>348</v>
-      </c>
-      <c r="R31" s="7" t="s">
+      <c r="P31" s="13" t="s">
+        <v>47</v>
+      </c>
+      <c r="Q31" s="14" t="s">
+        <v>347</v>
+      </c>
+      <c r="R31" s="21" t="s">
         <v>342</v>
       </c>
     </row>
-    <row r="32" spans="1:20" ht="45" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:19" ht="45" x14ac:dyDescent="0.25">
       <c r="A32" s="3">
         <v>2</v>
       </c>

</xml_diff>

<commit_message>
- changed 7499110123 (X4) to 30726 out of TE.DbLib/CON_IO - adjusted voltage rating of caps for power supply:      220uF (C48,C49,C58,C59,C68,C69,C86) to 23410 out of TE.DbLib/C_2012_0805      47uF (C92,C93) to 24718 out of TE.DbLib/C_2012_0805
</commit_message>
<xml_diff>
--- a/Using Trenz Library/BOM_MissingComponents_in_process_Simon.xlsx
+++ b/Using Trenz Library/BOM_MissingComponents_in_process_Simon.xlsx
@@ -1232,7 +1232,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1282,6 +1282,9 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -3218,7 +3221,7 @@
         <v>334</v>
       </c>
     </row>
-    <row r="33" spans="1:17" ht="45" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:19" ht="45" x14ac:dyDescent="0.25">
       <c r="A33" s="3">
         <v>4</v>
       </c>
@@ -3265,7 +3268,7 @@
         <v>334</v>
       </c>
     </row>
-    <row r="34" spans="1:17" ht="30" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:19" ht="30" x14ac:dyDescent="0.25">
       <c r="A34" s="3">
         <v>4</v>
       </c>
@@ -3310,7 +3313,7 @@
         <v>334</v>
       </c>
     </row>
-    <row r="35" spans="1:17" ht="30" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:19" ht="30" x14ac:dyDescent="0.25">
       <c r="A35" s="3">
         <v>1</v>
       </c>
@@ -3357,7 +3360,7 @@
         <v>323</v>
       </c>
     </row>
-    <row r="36" spans="1:17" ht="45" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:19" ht="45" x14ac:dyDescent="0.25">
       <c r="A36" s="3">
         <v>1</v>
       </c>
@@ -3408,7 +3411,7 @@
         <v>323</v>
       </c>
     </row>
-    <row r="37" spans="1:17" ht="45" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:19" ht="45" x14ac:dyDescent="0.25">
       <c r="A37" s="3">
         <v>1</v>
       </c>
@@ -3459,7 +3462,7 @@
         <v>323</v>
       </c>
     </row>
-    <row r="38" spans="1:17" ht="45" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:19" ht="45" x14ac:dyDescent="0.25">
       <c r="A38" s="3">
         <v>1</v>
       </c>
@@ -3510,7 +3513,7 @@
         <v>323</v>
       </c>
     </row>
-    <row r="39" spans="1:17" ht="45" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:19" ht="45" x14ac:dyDescent="0.25">
       <c r="A39" s="3">
         <v>1</v>
       </c>
@@ -3561,7 +3564,7 @@
         <v>323</v>
       </c>
     </row>
-    <row r="40" spans="1:17" ht="45" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:19" ht="45" x14ac:dyDescent="0.25">
       <c r="A40" s="3">
         <v>1</v>
       </c>
@@ -3612,60 +3615,62 @@
         <v>323</v>
       </c>
     </row>
-    <row r="41" spans="1:17" ht="45" x14ac:dyDescent="0.25">
-      <c r="A41" s="3">
+    <row r="41" spans="1:19" ht="45" x14ac:dyDescent="0.25">
+      <c r="A41" s="12">
         <v>1</v>
       </c>
-      <c r="B41" s="4" t="s">
+      <c r="B41" s="13" t="s">
         <v>56</v>
       </c>
-      <c r="C41" s="4" t="s">
+      <c r="C41" s="13" t="s">
         <v>57</v>
       </c>
-      <c r="D41" s="4" t="s">
+      <c r="D41" s="13" t="s">
         <v>58</v>
       </c>
-      <c r="E41" s="4" t="s">
+      <c r="E41" s="13" t="s">
         <v>56</v>
       </c>
-      <c r="F41" s="4" t="s">
+      <c r="F41" s="13" t="s">
         <v>56</v>
       </c>
-      <c r="G41" s="4" t="s">
+      <c r="G41" s="13" t="s">
         <v>59</v>
       </c>
-      <c r="H41" s="4" t="s">
+      <c r="H41" s="13" t="s">
         <v>56</v>
       </c>
-      <c r="I41" s="4" t="s">
+      <c r="I41" s="13" t="s">
         <v>60</v>
       </c>
-      <c r="J41" s="4" t="s">
+      <c r="J41" s="13" t="s">
         <v>23</v>
       </c>
-      <c r="K41" s="4" t="s">
+      <c r="K41" s="13" t="s">
         <v>61</v>
       </c>
-      <c r="L41" s="4" t="s">
+      <c r="L41" s="13" t="s">
         <v>25</v>
       </c>
-      <c r="M41" s="4" t="s">
+      <c r="M41" s="13" t="s">
         <v>62</v>
       </c>
-      <c r="N41" s="4" t="s">
+      <c r="N41" s="13" t="s">
         <v>36</v>
       </c>
-      <c r="O41" s="4" t="s">
+      <c r="O41" s="13" t="s">
         <v>63</v>
       </c>
-      <c r="P41" s="4" t="s">
-        <v>47</v>
-      </c>
-      <c r="Q41" s="5" t="s">
+      <c r="P41" s="13" t="s">
+        <v>47</v>
+      </c>
+      <c r="Q41" s="22" t="s">
         <v>325</v>
       </c>
-    </row>
-    <row r="42" spans="1:17" ht="60" x14ac:dyDescent="0.25">
+      <c r="R41" s="16"/>
+      <c r="S41" s="15"/>
+    </row>
+    <row r="42" spans="1:19" ht="60" x14ac:dyDescent="0.25">
       <c r="A42" s="3">
         <v>3</v>
       </c>
@@ -3716,7 +3721,7 @@
         <v>323</v>
       </c>
     </row>
-    <row r="43" spans="1:17" ht="60" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:19" ht="60" x14ac:dyDescent="0.25">
       <c r="A43" s="3">
         <v>5</v>
       </c>
@@ -3767,7 +3772,7 @@
         <v>323</v>
       </c>
     </row>
-    <row r="44" spans="1:17" ht="45" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:19" ht="45" x14ac:dyDescent="0.25">
       <c r="A44" s="3">
         <v>2</v>
       </c>

</xml_diff>

<commit_message>
adjusted votlage rating of caps for power supply: 10uF 35V to 24685 (10uF 50V) out of TE.DbLib/C_3216_1206 (changed PCB layout of power supply)
</commit_message>
<xml_diff>
--- a/Using Trenz Library/BOM_MissingComponents_in_process_Simon.xlsx
+++ b/Using Trenz Library/BOM_MissingComponents_in_process_Simon.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="638" uniqueCount="358">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="638" uniqueCount="360">
   <si>
     <t>Quantity</t>
   </si>
@@ -1101,6 +1101,12 @@
   </si>
   <si>
     <t>used 29707</t>
+  </si>
+  <si>
+    <t>ISO7741QDWRQ1                                                      Mouser: 595-ISO7741QDWRQ1</t>
+  </si>
+  <si>
+    <t>ISO7742QDWRQ1                                                  Mouser:595-ISO7742QDWRQ1</t>
   </si>
 </sst>
 </file>
@@ -1232,7 +1238,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1286,6 +1292,7 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Link" xfId="1" builtinId="8"/>
@@ -1588,7 +1595,7 @@
     <col min="14" max="14" width="7.28515625" customWidth="1"/>
     <col min="15" max="15" width="9.85546875" customWidth="1"/>
     <col min="16" max="16" width="16" customWidth="1"/>
-    <col min="17" max="17" width="40.140625" customWidth="1"/>
+    <col min="17" max="17" width="42.140625" customWidth="1"/>
     <col min="18" max="18" width="24.42578125" style="7" customWidth="1"/>
     <col min="19" max="19" width="14.140625" customWidth="1"/>
   </cols>
@@ -1690,7 +1697,7 @@
       <c r="P2" s="4" t="s">
         <v>47</v>
       </c>
-      <c r="Q2" s="10" t="s">
+      <c r="Q2" s="23" t="s">
         <v>320</v>
       </c>
       <c r="R2" s="7" t="s">
@@ -2900,7 +2907,7 @@
         <v>47</v>
       </c>
       <c r="Q26" s="5" t="s">
-        <v>346</v>
+        <v>358</v>
       </c>
       <c r="R26" s="7" t="s">
         <v>348</v>
@@ -3003,8 +3010,8 @@
       <c r="P28" s="4" t="s">
         <v>47</v>
       </c>
-      <c r="Q28" t="s">
-        <v>346</v>
+      <c r="Q28" s="7" t="s">
+        <v>359</v>
       </c>
       <c r="R28" s="7" t="s">
         <v>348</v>

</xml_diff>

<commit_message>
changed IPL1-110-02-L-D-K (X3) to 30765 out of TE.DbLib/CON_HEADER, IPL1-106-02-L-D-K (X10) to 30763 out of TE.DbLib/CON_HEADER, HSEC8-140-01-L-DV-A-BL (X5) to 30758 (HTEC8-140-01-L-DV-K) out of TE.DbLib/CON_B2B
</commit_message>
<xml_diff>
--- a/Using Trenz Library/BOM_MissingComponents_in_process_Simon.xlsx
+++ b/Using Trenz Library/BOM_MissingComponents_in_process_Simon.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="638" uniqueCount="360">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="643" uniqueCount="362">
   <si>
     <t>Quantity</t>
   </si>
@@ -1107,6 +1107,12 @@
   </si>
   <si>
     <t>ISO7742QDWRQ1                                                  Mouser:595-ISO7742QDWRQ1</t>
+  </si>
+  <si>
+    <t>used SMD (02) connector</t>
+  </si>
+  <si>
+    <t>used HTEC8-140-01-L-DV-K</t>
   </si>
 </sst>
 </file>
@@ -1238,7 +1244,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="26">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1293,6 +1299,12 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Link" xfId="1" builtinId="8"/>
@@ -3321,306 +3333,326 @@
       </c>
     </row>
     <row r="35" spans="1:19" ht="30" x14ac:dyDescent="0.25">
-      <c r="A35" s="3">
+      <c r="A35" s="12">
         <v>1</v>
       </c>
-      <c r="B35" s="4" t="s">
+      <c r="B35" s="13" t="s">
         <v>102</v>
       </c>
-      <c r="C35" s="4" t="s">
+      <c r="C35" s="13" t="s">
         <v>103</v>
       </c>
-      <c r="D35" s="4" t="s">
+      <c r="D35" s="13" t="s">
         <v>86</v>
       </c>
-      <c r="E35" s="4" t="s">
+      <c r="E35" s="13" t="s">
         <v>102</v>
       </c>
-      <c r="F35" s="4" t="s">
+      <c r="F35" s="13" t="s">
         <v>102</v>
       </c>
-      <c r="G35" s="4" t="s">
+      <c r="G35" s="13" t="s">
         <v>87</v>
       </c>
-      <c r="H35" s="4" t="s">
+      <c r="H35" s="13" t="s">
         <v>102</v>
       </c>
-      <c r="I35" s="3"/>
-      <c r="J35" s="4" t="s">
+      <c r="I35" s="12"/>
+      <c r="J35" s="13" t="s">
         <v>25</v>
       </c>
-      <c r="K35" s="4" t="s">
+      <c r="K35" s="13" t="s">
         <v>104</v>
       </c>
-      <c r="L35" s="4" t="s">
+      <c r="L35" s="13" t="s">
         <v>36</v>
       </c>
-      <c r="M35" s="4" t="s">
+      <c r="M35" s="13" t="s">
         <v>105</v>
       </c>
-      <c r="N35" s="3"/>
-      <c r="O35" s="3"/>
-      <c r="P35" s="4" t="s">
-        <v>47</v>
-      </c>
-      <c r="Q35" s="5" t="s">
+      <c r="N35" s="12"/>
+      <c r="O35" s="12"/>
+      <c r="P35" s="13" t="s">
+        <v>47</v>
+      </c>
+      <c r="Q35" s="22" t="s">
         <v>323</v>
       </c>
+      <c r="R35" s="16"/>
+      <c r="S35" s="15"/>
     </row>
     <row r="36" spans="1:19" ht="45" x14ac:dyDescent="0.25">
-      <c r="A36" s="3">
+      <c r="A36" s="12">
         <v>1</v>
       </c>
-      <c r="B36" s="4" t="s">
+      <c r="B36" s="13" t="s">
         <v>91</v>
       </c>
-      <c r="C36" s="4" t="s">
+      <c r="C36" s="13" t="s">
         <v>92</v>
       </c>
-      <c r="D36" s="4" t="s">
+      <c r="D36" s="13" t="s">
         <v>86</v>
       </c>
-      <c r="E36" s="4" t="s">
+      <c r="E36" s="13" t="s">
         <v>91</v>
       </c>
-      <c r="F36" s="4" t="s">
+      <c r="F36" s="13" t="s">
         <v>91</v>
       </c>
-      <c r="G36" s="4" t="s">
+      <c r="G36" s="13" t="s">
         <v>93</v>
       </c>
-      <c r="H36" s="4" t="s">
+      <c r="H36" s="13" t="s">
         <v>91</v>
       </c>
-      <c r="I36" s="3"/>
-      <c r="J36" s="4" t="s">
+      <c r="I36" s="12"/>
+      <c r="J36" s="13" t="s">
         <v>23</v>
       </c>
-      <c r="K36" s="4" t="s">
+      <c r="K36" s="13" t="s">
         <v>94</v>
       </c>
-      <c r="L36" s="4" t="s">
+      <c r="L36" s="13" t="s">
         <v>25</v>
       </c>
-      <c r="M36" s="4" t="s">
+      <c r="M36" s="13" t="s">
         <v>95</v>
       </c>
-      <c r="N36" s="4" t="s">
+      <c r="N36" s="13" t="s">
         <v>36</v>
       </c>
-      <c r="O36" s="4" t="s">
+      <c r="O36" s="13" t="s">
         <v>96</v>
       </c>
-      <c r="P36" s="4" t="s">
-        <v>47</v>
-      </c>
-      <c r="Q36" s="5" t="s">
+      <c r="P36" s="13" t="s">
+        <v>47</v>
+      </c>
+      <c r="Q36" s="22" t="s">
         <v>323</v>
       </c>
+      <c r="R36" s="16"/>
+      <c r="S36" s="24" t="s">
+        <v>360</v>
+      </c>
     </row>
     <row r="37" spans="1:19" ht="45" x14ac:dyDescent="0.25">
-      <c r="A37" s="3">
+      <c r="A37" s="12">
         <v>1</v>
       </c>
-      <c r="B37" s="4" t="s">
+      <c r="B37" s="13" t="s">
         <v>106</v>
       </c>
-      <c r="C37" s="4" t="s">
+      <c r="C37" s="13" t="s">
         <v>107</v>
       </c>
-      <c r="D37" s="4" t="s">
+      <c r="D37" s="13" t="s">
         <v>86</v>
       </c>
-      <c r="E37" s="4" t="s">
+      <c r="E37" s="13" t="s">
         <v>106</v>
       </c>
-      <c r="F37" s="4" t="s">
+      <c r="F37" s="13" t="s">
         <v>106</v>
       </c>
-      <c r="G37" s="4" t="s">
+      <c r="G37" s="13" t="s">
         <v>93</v>
       </c>
-      <c r="H37" s="4" t="s">
+      <c r="H37" s="13" t="s">
         <v>106</v>
       </c>
-      <c r="I37" s="3"/>
-      <c r="J37" s="4" t="s">
+      <c r="I37" s="12"/>
+      <c r="J37" s="13" t="s">
         <v>23</v>
       </c>
-      <c r="K37" s="4" t="s">
+      <c r="K37" s="13" t="s">
         <v>108</v>
       </c>
-      <c r="L37" s="4" t="s">
+      <c r="L37" s="13" t="s">
         <v>25</v>
       </c>
-      <c r="M37" s="4" t="s">
+      <c r="M37" s="13" t="s">
         <v>109</v>
       </c>
-      <c r="N37" s="4" t="s">
+      <c r="N37" s="13" t="s">
         <v>36</v>
       </c>
-      <c r="O37" s="4" t="s">
+      <c r="O37" s="13" t="s">
         <v>110</v>
       </c>
-      <c r="P37" s="4" t="s">
-        <v>47</v>
-      </c>
-      <c r="Q37" s="5" t="s">
+      <c r="P37" s="13" t="s">
+        <v>47</v>
+      </c>
+      <c r="Q37" s="22" t="s">
         <v>323</v>
       </c>
+      <c r="R37" s="16"/>
+      <c r="S37" s="24" t="s">
+        <v>360</v>
+      </c>
     </row>
     <row r="38" spans="1:19" ht="45" x14ac:dyDescent="0.25">
-      <c r="A38" s="3">
+      <c r="A38" s="12">
         <v>1</v>
       </c>
-      <c r="B38" s="4" t="s">
+      <c r="B38" s="13" t="s">
         <v>97</v>
       </c>
-      <c r="C38" s="4" t="s">
+      <c r="C38" s="13" t="s">
         <v>98</v>
       </c>
-      <c r="D38" s="4" t="s">
+      <c r="D38" s="13" t="s">
         <v>86</v>
       </c>
-      <c r="E38" s="4" t="s">
+      <c r="E38" s="13" t="s">
         <v>97</v>
       </c>
-      <c r="F38" s="4" t="s">
+      <c r="F38" s="13" t="s">
         <v>97</v>
       </c>
-      <c r="G38" s="4" t="s">
+      <c r="G38" s="13" t="s">
         <v>93</v>
       </c>
-      <c r="H38" s="4" t="s">
+      <c r="H38" s="13" t="s">
         <v>97</v>
       </c>
-      <c r="I38" s="3"/>
-      <c r="J38" s="4" t="s">
+      <c r="I38" s="12"/>
+      <c r="J38" s="13" t="s">
         <v>23</v>
       </c>
-      <c r="K38" s="4" t="s">
+      <c r="K38" s="13" t="s">
         <v>99</v>
       </c>
-      <c r="L38" s="4" t="s">
+      <c r="L38" s="13" t="s">
         <v>25</v>
       </c>
-      <c r="M38" s="4" t="s">
+      <c r="M38" s="13" t="s">
         <v>100</v>
       </c>
-      <c r="N38" s="4" t="s">
+      <c r="N38" s="13" t="s">
         <v>36</v>
       </c>
-      <c r="O38" s="4" t="s">
+      <c r="O38" s="13" t="s">
         <v>101</v>
       </c>
-      <c r="P38" s="4" t="s">
-        <v>47</v>
-      </c>
-      <c r="Q38" s="5" t="s">
+      <c r="P38" s="13" t="s">
+        <v>47</v>
+      </c>
+      <c r="Q38" s="22" t="s">
         <v>323</v>
       </c>
+      <c r="R38" s="16"/>
+      <c r="S38" s="24" t="s">
+        <v>360</v>
+      </c>
     </row>
     <row r="39" spans="1:19" ht="45" x14ac:dyDescent="0.25">
-      <c r="A39" s="3">
+      <c r="A39" s="12">
         <v>1</v>
       </c>
-      <c r="B39" s="4" t="s">
+      <c r="B39" s="13" t="s">
         <v>84</v>
       </c>
-      <c r="C39" s="4" t="s">
+      <c r="C39" s="13" t="s">
         <v>85</v>
       </c>
-      <c r="D39" s="4" t="s">
+      <c r="D39" s="13" t="s">
         <v>86</v>
       </c>
-      <c r="E39" s="4" t="s">
+      <c r="E39" s="13" t="s">
         <v>84</v>
       </c>
-      <c r="F39" s="4" t="s">
+      <c r="F39" s="13" t="s">
         <v>84</v>
       </c>
-      <c r="G39" s="4" t="s">
+      <c r="G39" s="13" t="s">
         <v>87</v>
       </c>
-      <c r="H39" s="4" t="s">
+      <c r="H39" s="13" t="s">
         <v>84</v>
       </c>
-      <c r="I39" s="3"/>
-      <c r="J39" s="4" t="s">
+      <c r="I39" s="12"/>
+      <c r="J39" s="13" t="s">
         <v>23</v>
       </c>
-      <c r="K39" s="4" t="s">
+      <c r="K39" s="13" t="s">
         <v>88</v>
       </c>
-      <c r="L39" s="4" t="s">
+      <c r="L39" s="13" t="s">
         <v>25</v>
       </c>
-      <c r="M39" s="4" t="s">
+      <c r="M39" s="13" t="s">
         <v>89</v>
       </c>
-      <c r="N39" s="4" t="s">
+      <c r="N39" s="13" t="s">
         <v>36</v>
       </c>
-      <c r="O39" s="4" t="s">
+      <c r="O39" s="13" t="s">
         <v>90</v>
       </c>
-      <c r="P39" s="4" t="s">
-        <v>47</v>
-      </c>
-      <c r="Q39" s="5" t="s">
+      <c r="P39" s="13" t="s">
+        <v>47</v>
+      </c>
+      <c r="Q39" s="22" t="s">
         <v>323</v>
       </c>
+      <c r="R39" s="16"/>
+      <c r="S39" s="24" t="s">
+        <v>360</v>
+      </c>
     </row>
     <row r="40" spans="1:19" ht="45" x14ac:dyDescent="0.25">
-      <c r="A40" s="3">
+      <c r="A40" s="12">
         <v>1</v>
       </c>
-      <c r="B40" s="4" t="s">
+      <c r="B40" s="13" t="s">
         <v>111</v>
       </c>
-      <c r="C40" s="4" t="s">
+      <c r="C40" s="13" t="s">
         <v>112</v>
       </c>
-      <c r="D40" s="4" t="s">
+      <c r="D40" s="13" t="s">
         <v>86</v>
       </c>
-      <c r="E40" s="4" t="s">
+      <c r="E40" s="13" t="s">
         <v>111</v>
       </c>
-      <c r="F40" s="4" t="s">
+      <c r="F40" s="13" t="s">
         <v>111</v>
       </c>
-      <c r="G40" s="4" t="s">
+      <c r="G40" s="13" t="s">
         <v>93</v>
       </c>
-      <c r="H40" s="4" t="s">
+      <c r="H40" s="13" t="s">
         <v>111</v>
       </c>
-      <c r="I40" s="3"/>
-      <c r="J40" s="4" t="s">
+      <c r="I40" s="12"/>
+      <c r="J40" s="13" t="s">
         <v>23</v>
       </c>
-      <c r="K40" s="4" t="s">
+      <c r="K40" s="13" t="s">
         <v>113</v>
       </c>
-      <c r="L40" s="4" t="s">
+      <c r="L40" s="13" t="s">
         <v>25</v>
       </c>
-      <c r="M40" s="4" t="s">
+      <c r="M40" s="13" t="s">
         <v>114</v>
       </c>
-      <c r="N40" s="4" t="s">
+      <c r="N40" s="13" t="s">
         <v>36</v>
       </c>
-      <c r="O40" s="4" t="s">
+      <c r="O40" s="13" t="s">
         <v>115</v>
       </c>
-      <c r="P40" s="4" t="s">
-        <v>47</v>
-      </c>
-      <c r="Q40" s="5" t="s">
+      <c r="P40" s="13" t="s">
+        <v>47</v>
+      </c>
+      <c r="Q40" s="22" t="s">
         <v>323</v>
       </c>
+      <c r="R40" s="16"/>
+      <c r="S40" s="15"/>
     </row>
     <row r="41" spans="1:19" ht="45" x14ac:dyDescent="0.25">
       <c r="A41" s="12">
@@ -3681,51 +3713,55 @@
       <c r="A42" s="3">
         <v>3</v>
       </c>
-      <c r="B42" s="4" t="s">
+      <c r="B42" s="13" t="s">
         <v>217</v>
       </c>
-      <c r="C42" s="4" t="s">
+      <c r="C42" s="13" t="s">
         <v>218</v>
       </c>
-      <c r="D42" s="4" t="s">
+      <c r="D42" s="13" t="s">
         <v>86</v>
       </c>
-      <c r="E42" s="4" t="s">
+      <c r="E42" s="13" t="s">
         <v>217</v>
       </c>
-      <c r="F42" s="4" t="s">
+      <c r="F42" s="13" t="s">
         <v>217</v>
       </c>
-      <c r="G42" s="4" t="s">
+      <c r="G42" s="13" t="s">
         <v>219</v>
       </c>
-      <c r="H42" s="4" t="s">
+      <c r="H42" s="13" t="s">
         <v>220</v>
       </c>
-      <c r="I42" s="3"/>
-      <c r="J42" s="4" t="s">
+      <c r="I42" s="12"/>
+      <c r="J42" s="13" t="s">
         <v>23</v>
       </c>
-      <c r="K42" s="4" t="s">
+      <c r="K42" s="13" t="s">
         <v>221</v>
       </c>
-      <c r="L42" s="4" t="s">
+      <c r="L42" s="13" t="s">
         <v>25</v>
       </c>
-      <c r="M42" s="4" t="s">
+      <c r="M42" s="13" t="s">
         <v>222</v>
       </c>
-      <c r="N42" s="4" t="s">
+      <c r="N42" s="13" t="s">
         <v>36</v>
       </c>
-      <c r="O42" s="4" t="s">
+      <c r="O42" s="13" t="s">
         <v>223</v>
       </c>
-      <c r="P42" s="4" t="s">
-        <v>47</v>
-      </c>
-      <c r="Q42" s="5" t="s">
+      <c r="P42" s="13" t="s">
+        <v>47</v>
+      </c>
+      <c r="Q42" s="22" t="s">
         <v>323</v>
+      </c>
+      <c r="R42" s="16"/>
+      <c r="S42" s="25" t="s">
+        <v>361</v>
       </c>
     </row>
     <row r="43" spans="1:19" ht="60" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
changed HSEC8-150-01-L-DV-A-BL (X6) to 30757 (HTEC8-150-01-L-DV-K)  out of TE.DbLib/CON_B2B
</commit_message>
<xml_diff>
--- a/Using Trenz Library/BOM_MissingComponents_in_process_Simon.xlsx
+++ b/Using Trenz Library/BOM_MissingComponents_in_process_Simon.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="643" uniqueCount="362">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="644" uniqueCount="363">
   <si>
     <t>Quantity</t>
   </si>
@@ -1113,6 +1113,9 @@
   </si>
   <si>
     <t>used HTEC8-140-01-L-DV-K</t>
+  </si>
+  <si>
+    <t>used HTEC8-150-01-L-DV-K</t>
   </si>
 </sst>
 </file>
@@ -3768,51 +3771,55 @@
       <c r="A43" s="3">
         <v>5</v>
       </c>
-      <c r="B43" s="4" t="s">
+      <c r="B43" s="13" t="s">
         <v>262</v>
       </c>
-      <c r="C43" s="4" t="s">
+      <c r="C43" s="13" t="s">
         <v>263</v>
       </c>
-      <c r="D43" s="4" t="s">
+      <c r="D43" s="13" t="s">
         <v>86</v>
       </c>
-      <c r="E43" s="4" t="s">
+      <c r="E43" s="13" t="s">
         <v>262</v>
       </c>
-      <c r="F43" s="4" t="s">
+      <c r="F43" s="13" t="s">
         <v>262</v>
       </c>
-      <c r="G43" s="4" t="s">
+      <c r="G43" s="13" t="s">
         <v>219</v>
       </c>
-      <c r="H43" s="4" t="s">
+      <c r="H43" s="13" t="s">
         <v>264</v>
       </c>
-      <c r="I43" s="3"/>
-      <c r="J43" s="4" t="s">
+      <c r="I43" s="12"/>
+      <c r="J43" s="13" t="s">
         <v>23</v>
       </c>
-      <c r="K43" s="4" t="s">
+      <c r="K43" s="13" t="s">
         <v>265</v>
       </c>
-      <c r="L43" s="4" t="s">
+      <c r="L43" s="13" t="s">
         <v>25</v>
       </c>
-      <c r="M43" s="4" t="s">
+      <c r="M43" s="13" t="s">
         <v>266</v>
       </c>
-      <c r="N43" s="4" t="s">
+      <c r="N43" s="13" t="s">
         <v>36</v>
       </c>
-      <c r="O43" s="4" t="s">
+      <c r="O43" s="13" t="s">
         <v>267</v>
       </c>
-      <c r="P43" s="4" t="s">
-        <v>47</v>
-      </c>
-      <c r="Q43" s="5" t="s">
+      <c r="P43" s="13" t="s">
+        <v>47</v>
+      </c>
+      <c r="Q43" s="22" t="s">
         <v>323</v>
+      </c>
+      <c r="R43" s="16"/>
+      <c r="S43" s="25" t="s">
+        <v>362</v>
       </c>
     </row>
     <row r="44" spans="1:19" ht="45" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
changed ADUM4401 (U18) to 30781 (ISO7741QDWRQ1) out of TE.DbLib/SPECIAL
</commit_message>
<xml_diff>
--- a/Using Trenz Library/BOM_MissingComponents_in_process_Simon.xlsx
+++ b/Using Trenz Library/BOM_MissingComponents_in_process_Simon.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="644" uniqueCount="363">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="645" uniqueCount="364">
   <si>
     <t>Quantity</t>
   </si>
@@ -1116,6 +1116,9 @@
   </si>
   <si>
     <t>used HTEC8-150-01-L-DV-K</t>
+  </si>
+  <si>
+    <t>used ISO7741QDWRQ1</t>
   </si>
 </sst>
 </file>
@@ -2880,52 +2883,55 @@
       <c r="A26" s="3">
         <v>1</v>
       </c>
-      <c r="B26" s="4" t="s">
+      <c r="B26" s="13" t="s">
         <v>64</v>
       </c>
-      <c r="C26" s="4" t="s">
+      <c r="C26" s="13" t="s">
         <v>65</v>
       </c>
-      <c r="D26" s="4" t="s">
+      <c r="D26" s="13" t="s">
         <v>66</v>
       </c>
-      <c r="E26" s="4" t="s">
+      <c r="E26" s="13" t="s">
         <v>67</v>
       </c>
-      <c r="F26" s="4" t="s">
+      <c r="F26" s="13" t="s">
         <v>64</v>
       </c>
-      <c r="G26" s="4" t="s">
+      <c r="G26" s="13" t="s">
         <v>68</v>
       </c>
-      <c r="H26" s="4" t="s">
+      <c r="H26" s="13" t="s">
         <v>69</v>
       </c>
-      <c r="I26" s="4" t="s">
+      <c r="I26" s="13" t="s">
         <v>70</v>
       </c>
-      <c r="J26" s="4" t="s">
+      <c r="J26" s="13" t="s">
         <v>25</v>
       </c>
-      <c r="K26" s="4" t="s">
+      <c r="K26" s="13" t="s">
         <v>71</v>
       </c>
-      <c r="L26" s="4" t="s">
+      <c r="L26" s="13" t="s">
         <v>72</v>
       </c>
-      <c r="M26" s="4" t="s">
+      <c r="M26" s="13" t="s">
         <v>73</v>
       </c>
-      <c r="N26" s="3"/>
-      <c r="O26" s="3"/>
-      <c r="P26" s="4" t="s">
-        <v>47</v>
-      </c>
-      <c r="Q26" s="5" t="s">
+      <c r="N26" s="12"/>
+      <c r="O26" s="12"/>
+      <c r="P26" s="13" t="s">
+        <v>47</v>
+      </c>
+      <c r="Q26" s="22" t="s">
         <v>358</v>
       </c>
-      <c r="R26" s="7" t="s">
+      <c r="R26" s="16" t="s">
         <v>348</v>
+      </c>
+      <c r="S26" s="24" t="s">
+        <v>363</v>
       </c>
     </row>
     <row r="27" spans="1:19" ht="90" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
changed ADUM4402 (U24,U26) to 30782 (ISO7742QDWRQ1) out of TE.DbLib/SPECIAL
</commit_message>
<xml_diff>
--- a/Using Trenz Library/BOM_MissingComponents_in_process_Simon.xlsx
+++ b/Using Trenz Library/BOM_MissingComponents_in_process_Simon.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="645" uniqueCount="364">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="646" uniqueCount="365">
   <si>
     <t>Quantity</t>
   </si>
@@ -1119,6 +1119,9 @@
   </si>
   <si>
     <t>used ISO7741QDWRQ1</t>
+  </si>
+  <si>
+    <t>used ISO7742QDWRQ1</t>
   </si>
 </sst>
 </file>
@@ -2994,48 +2997,51 @@
       <c r="A28" s="3">
         <v>2</v>
       </c>
-      <c r="B28" s="4" t="s">
+      <c r="B28" s="13" t="s">
         <v>169</v>
       </c>
-      <c r="C28" s="4" t="s">
+      <c r="C28" s="13" t="s">
         <v>170</v>
       </c>
-      <c r="D28" s="4" t="s">
+      <c r="D28" s="13" t="s">
         <v>66</v>
       </c>
-      <c r="E28" s="4" t="s">
+      <c r="E28" s="13" t="s">
         <v>171</v>
       </c>
-      <c r="F28" s="4" t="s">
+      <c r="F28" s="13" t="s">
         <v>169</v>
       </c>
-      <c r="G28" s="4" t="s">
+      <c r="G28" s="13" t="s">
         <v>172</v>
       </c>
-      <c r="H28" s="4" t="s">
+      <c r="H28" s="13" t="s">
         <v>69</v>
       </c>
-      <c r="I28" s="4" t="s">
+      <c r="I28" s="13" t="s">
         <v>70</v>
       </c>
-      <c r="J28" s="4" t="s">
+      <c r="J28" s="13" t="s">
         <v>25</v>
       </c>
-      <c r="K28" s="4" t="s">
+      <c r="K28" s="13" t="s">
         <v>173</v>
       </c>
-      <c r="L28" s="3"/>
-      <c r="M28" s="3"/>
-      <c r="N28" s="3"/>
-      <c r="O28" s="3"/>
-      <c r="P28" s="4" t="s">
-        <v>47</v>
-      </c>
-      <c r="Q28" s="7" t="s">
+      <c r="L28" s="12"/>
+      <c r="M28" s="12"/>
+      <c r="N28" s="12"/>
+      <c r="O28" s="12"/>
+      <c r="P28" s="13" t="s">
+        <v>47</v>
+      </c>
+      <c r="Q28" s="16" t="s">
         <v>359</v>
       </c>
-      <c r="R28" s="7" t="s">
+      <c r="R28" s="16" t="s">
         <v>348</v>
+      </c>
+      <c r="S28" s="17" t="s">
+        <v>364</v>
       </c>
     </row>
     <row r="29" spans="1:19" ht="60" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
changed MAX14878AWE+ (U6) to 30766 out of TE.DbLib/IF, LMK00105SQ/NOPB (U32) to 30774 out of TE.DbLib/CLK
</commit_message>
<xml_diff>
--- a/Using Trenz Library/BOM_MissingComponents_in_process_Simon.xlsx
+++ b/Using Trenz Library/BOM_MissingComponents_in_process_Simon.xlsx
@@ -1253,7 +1253,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="26">
+  <cellXfs count="27">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1312,6 +1312,9 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -2883,7 +2886,7 @@
       </c>
     </row>
     <row r="26" spans="1:19" ht="45" x14ac:dyDescent="0.25">
-      <c r="A26" s="3">
+      <c r="A26" s="12">
         <v>1</v>
       </c>
       <c r="B26" s="13" t="s">
@@ -2994,7 +2997,7 @@
       </c>
     </row>
     <row r="28" spans="1:19" ht="45" x14ac:dyDescent="0.25">
-      <c r="A28" s="3">
+      <c r="A28" s="12">
         <v>2</v>
       </c>
       <c r="B28" s="13" t="s">
@@ -3045,57 +3048,59 @@
       </c>
     </row>
     <row r="29" spans="1:19" ht="60" x14ac:dyDescent="0.25">
-      <c r="A29" s="3">
+      <c r="A29" s="12">
         <v>1</v>
       </c>
-      <c r="B29" s="4" t="s">
+      <c r="B29" s="13" t="s">
         <v>116</v>
       </c>
-      <c r="C29" s="4" t="s">
+      <c r="C29" s="13" t="s">
         <v>117</v>
       </c>
-      <c r="D29" s="4" t="s">
+      <c r="D29" s="13" t="s">
         <v>118</v>
       </c>
-      <c r="E29" s="4" t="s">
+      <c r="E29" s="13" t="s">
         <v>119</v>
       </c>
-      <c r="F29" s="4" t="s">
+      <c r="F29" s="13" t="s">
         <v>116</v>
       </c>
-      <c r="G29" s="4" t="s">
+      <c r="G29" s="13" t="s">
         <v>120</v>
       </c>
-      <c r="H29" s="4" t="s">
+      <c r="H29" s="13" t="s">
         <v>121</v>
       </c>
-      <c r="I29" s="4" t="s">
+      <c r="I29" s="13" t="s">
         <v>122</v>
       </c>
-      <c r="J29" s="4" t="s">
+      <c r="J29" s="13" t="s">
         <v>23</v>
       </c>
-      <c r="K29" s="4" t="s">
+      <c r="K29" s="13" t="s">
         <v>123</v>
       </c>
-      <c r="L29" s="4" t="s">
+      <c r="L29" s="13" t="s">
         <v>25</v>
       </c>
-      <c r="M29" s="4" t="s">
+      <c r="M29" s="13" t="s">
         <v>124</v>
       </c>
-      <c r="N29" s="4" t="s">
+      <c r="N29" s="13" t="s">
         <v>36</v>
       </c>
-      <c r="O29" s="4" t="s">
+      <c r="O29" s="13" t="s">
         <v>125</v>
       </c>
-      <c r="P29" s="4" t="s">
-        <v>47</v>
-      </c>
-      <c r="Q29" s="5" t="s">
+      <c r="P29" s="13" t="s">
+        <v>47</v>
+      </c>
+      <c r="Q29" s="22" t="s">
         <v>323</v>
       </c>
+      <c r="R29" s="16"/>
+      <c r="S29" s="15"/>
     </row>
     <row r="30" spans="1:19" ht="45" x14ac:dyDescent="0.25">
       <c r="A30" s="3">
@@ -3203,57 +3208,59 @@
       </c>
     </row>
     <row r="32" spans="1:19" ht="45" x14ac:dyDescent="0.25">
-      <c r="A32" s="3">
+      <c r="A32" s="12">
         <v>2</v>
       </c>
-      <c r="B32" s="4" t="s">
+      <c r="B32" s="13" t="s">
         <v>196</v>
       </c>
-      <c r="C32" s="4" t="s">
+      <c r="C32" s="13" t="s">
         <v>197</v>
       </c>
-      <c r="D32" s="4" t="s">
+      <c r="D32" s="13" t="s">
         <v>198</v>
       </c>
-      <c r="E32" s="4" t="s">
+      <c r="E32" s="13" t="s">
         <v>199</v>
       </c>
-      <c r="F32" s="4" t="s">
+      <c r="F32" s="13" t="s">
         <v>196</v>
       </c>
-      <c r="G32" s="4" t="s">
+      <c r="G32" s="13" t="s">
         <v>200</v>
       </c>
-      <c r="H32" s="4" t="s">
+      <c r="H32" s="13" t="s">
         <v>201</v>
       </c>
-      <c r="I32" s="4" t="s">
+      <c r="I32" s="13" t="s">
         <v>70</v>
       </c>
-      <c r="J32" s="4" t="s">
+      <c r="J32" s="13" t="s">
         <v>23</v>
       </c>
-      <c r="K32" s="4" t="s">
+      <c r="K32" s="13" t="s">
         <v>202</v>
       </c>
-      <c r="L32" s="4" t="s">
+      <c r="L32" s="13" t="s">
         <v>25</v>
       </c>
-      <c r="M32" s="4" t="s">
+      <c r="M32" s="13" t="s">
         <v>203</v>
       </c>
-      <c r="N32" s="4" t="s">
+      <c r="N32" s="13" t="s">
         <v>36</v>
       </c>
-      <c r="O32" s="4" t="s">
+      <c r="O32" s="13" t="s">
         <v>204</v>
       </c>
-      <c r="P32" s="4" t="s">
-        <v>47</v>
-      </c>
-      <c r="Q32" s="11" t="s">
+      <c r="P32" s="13" t="s">
+        <v>47</v>
+      </c>
+      <c r="Q32" s="26" t="s">
         <v>334</v>
       </c>
+      <c r="R32" s="16"/>
+      <c r="S32" s="15"/>
     </row>
     <row r="33" spans="1:19" ht="45" x14ac:dyDescent="0.25">
       <c r="A33" s="3">
@@ -3725,7 +3732,7 @@
       <c r="S41" s="15"/>
     </row>
     <row r="42" spans="1:19" ht="60" x14ac:dyDescent="0.25">
-      <c r="A42" s="3">
+      <c r="A42" s="12">
         <v>3</v>
       </c>
       <c r="B42" s="13" t="s">
@@ -3780,7 +3787,7 @@
       </c>
     </row>
     <row r="43" spans="1:19" ht="60" x14ac:dyDescent="0.25">
-      <c r="A43" s="3">
+      <c r="A43" s="12">
         <v>5</v>
       </c>
       <c r="B43" s="13" t="s">

</xml_diff>

<commit_message>
changed SN6505BDBVT (U9,U21,U29) to 30768 out of TE.DbLib/DRIVER, 76039015 (U8,U20,U28) to 30767 out of TE.DbLib/L_TRANS
</commit_message>
<xml_diff>
--- a/Using Trenz Library/BOM_MissingComponents_in_process_Simon.xlsx
+++ b/Using Trenz Library/BOM_MissingComponents_in_process_Simon.xlsx
@@ -1159,7 +1159,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1175,6 +1175,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FF92D050"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFF0000"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1279,9 +1285,6 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
@@ -1315,6 +1318,9 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" quotePrefix="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1721,7 +1727,7 @@
       <c r="P2" s="4" t="s">
         <v>47</v>
       </c>
-      <c r="Q2" s="23" t="s">
+      <c r="Q2" s="22" t="s">
         <v>320</v>
       </c>
       <c r="R2" s="7" t="s">
@@ -1729,114 +1735,114 @@
       </c>
     </row>
     <row r="3" spans="1:19" ht="45" x14ac:dyDescent="0.25">
-      <c r="A3" s="12">
+      <c r="A3" s="11">
         <v>6</v>
       </c>
-      <c r="B3" s="13" t="s">
+      <c r="B3" s="12" t="s">
         <v>276</v>
       </c>
-      <c r="C3" s="13" t="s">
+      <c r="C3" s="12" t="s">
         <v>277</v>
       </c>
-      <c r="D3" s="13" t="s">
+      <c r="D3" s="12" t="s">
         <v>58</v>
       </c>
-      <c r="E3" s="13" t="s">
+      <c r="E3" s="12" t="s">
         <v>276</v>
       </c>
-      <c r="F3" s="13" t="s">
+      <c r="F3" s="12" t="s">
         <v>276</v>
       </c>
-      <c r="G3" s="13" t="s">
+      <c r="G3" s="12" t="s">
         <v>278</v>
       </c>
-      <c r="H3" s="13" t="s">
+      <c r="H3" s="12" t="s">
         <v>158</v>
       </c>
-      <c r="I3" s="13" t="s">
+      <c r="I3" s="12" t="s">
         <v>54</v>
       </c>
-      <c r="J3" s="13" t="s">
+      <c r="J3" s="12" t="s">
         <v>23</v>
       </c>
-      <c r="K3" s="13" t="s">
+      <c r="K3" s="12" t="s">
         <v>279</v>
       </c>
-      <c r="L3" s="13" t="s">
+      <c r="L3" s="12" t="s">
         <v>25</v>
       </c>
-      <c r="M3" s="13" t="s">
+      <c r="M3" s="12" t="s">
         <v>280</v>
       </c>
-      <c r="N3" s="13" t="s">
+      <c r="N3" s="12" t="s">
         <v>36</v>
       </c>
-      <c r="O3" s="13" t="s">
+      <c r="O3" s="12" t="s">
         <v>281</v>
       </c>
-      <c r="P3" s="13" t="s">
-        <v>47</v>
-      </c>
-      <c r="Q3" s="14" t="s">
+      <c r="P3" s="12" t="s">
+        <v>47</v>
+      </c>
+      <c r="Q3" s="13" t="s">
         <v>321</v>
       </c>
-      <c r="R3" s="16"/>
-      <c r="S3" s="15"/>
+      <c r="R3" s="15"/>
+      <c r="S3" s="14"/>
     </row>
     <row r="4" spans="1:19" ht="45" x14ac:dyDescent="0.25">
-      <c r="A4" s="12">
+      <c r="A4" s="11">
         <v>2</v>
       </c>
-      <c r="B4" s="13" t="s">
+      <c r="B4" s="12" t="s">
         <v>155</v>
       </c>
-      <c r="C4" s="13" t="s">
+      <c r="C4" s="12" t="s">
         <v>156</v>
       </c>
-      <c r="D4" s="13" t="s">
+      <c r="D4" s="12" t="s">
         <v>58</v>
       </c>
-      <c r="E4" s="13" t="s">
+      <c r="E4" s="12" t="s">
         <v>155</v>
       </c>
-      <c r="F4" s="13" t="s">
+      <c r="F4" s="12" t="s">
         <v>155</v>
       </c>
-      <c r="G4" s="13" t="s">
+      <c r="G4" s="12" t="s">
         <v>157</v>
       </c>
-      <c r="H4" s="13" t="s">
+      <c r="H4" s="12" t="s">
         <v>158</v>
       </c>
-      <c r="I4" s="13" t="s">
+      <c r="I4" s="12" t="s">
         <v>54</v>
       </c>
-      <c r="J4" s="13" t="s">
+      <c r="J4" s="12" t="s">
         <v>23</v>
       </c>
-      <c r="K4" s="13" t="s">
+      <c r="K4" s="12" t="s">
         <v>159</v>
       </c>
-      <c r="L4" s="13" t="s">
+      <c r="L4" s="12" t="s">
         <v>25</v>
       </c>
-      <c r="M4" s="13" t="s">
+      <c r="M4" s="12" t="s">
         <v>160</v>
       </c>
-      <c r="N4" s="13" t="s">
+      <c r="N4" s="12" t="s">
         <v>36</v>
       </c>
-      <c r="O4" s="13" t="s">
+      <c r="O4" s="12" t="s">
         <v>161</v>
       </c>
-      <c r="P4" s="13" t="s">
-        <v>47</v>
-      </c>
-      <c r="Q4" s="14" t="s">
+      <c r="P4" s="12" t="s">
+        <v>47</v>
+      </c>
+      <c r="Q4" s="13" t="s">
         <v>322</v>
       </c>
-      <c r="R4" s="16"/>
-      <c r="S4" s="15"/>
+      <c r="R4" s="15"/>
+      <c r="S4" s="14"/>
     </row>
     <row r="5" spans="1:19" ht="45" x14ac:dyDescent="0.25">
       <c r="A5" s="3">
@@ -2004,102 +2010,102 @@
       </c>
     </row>
     <row r="8" spans="1:19" ht="30" x14ac:dyDescent="0.25">
-      <c r="A8" s="12">
+      <c r="A8" s="11">
         <v>1</v>
       </c>
-      <c r="B8" s="13" t="s">
+      <c r="B8" s="12" t="s">
         <v>134</v>
       </c>
-      <c r="C8" s="13" t="s">
+      <c r="C8" s="12" t="s">
         <v>135</v>
       </c>
-      <c r="D8" s="13" t="s">
+      <c r="D8" s="12" t="s">
         <v>136</v>
       </c>
-      <c r="E8" s="13" t="s">
+      <c r="E8" s="12" t="s">
         <v>137</v>
       </c>
-      <c r="F8" s="13" t="s">
+      <c r="F8" s="12" t="s">
         <v>134</v>
       </c>
-      <c r="G8" s="13" t="s">
+      <c r="G8" s="12" t="s">
         <v>138</v>
       </c>
-      <c r="H8" s="13" t="s">
+      <c r="H8" s="12" t="s">
         <v>139</v>
       </c>
-      <c r="I8" s="13" t="s">
+      <c r="I8" s="12" t="s">
         <v>140</v>
       </c>
-      <c r="J8" s="13" t="s">
+      <c r="J8" s="12" t="s">
         <v>25</v>
       </c>
-      <c r="K8" s="13" t="s">
+      <c r="K8" s="12" t="s">
         <v>141</v>
       </c>
-      <c r="L8" s="12"/>
-      <c r="M8" s="12"/>
-      <c r="N8" s="12"/>
-      <c r="O8" s="12"/>
-      <c r="P8" s="13" t="s">
-        <v>47</v>
-      </c>
-      <c r="Q8" s="15" t="s">
+      <c r="L8" s="11"/>
+      <c r="M8" s="11"/>
+      <c r="N8" s="11"/>
+      <c r="O8" s="11"/>
+      <c r="P8" s="12" t="s">
+        <v>47</v>
+      </c>
+      <c r="Q8" s="14" t="s">
         <v>350</v>
       </c>
-      <c r="R8" s="16"/>
-      <c r="S8" s="15"/>
+      <c r="R8" s="15"/>
+      <c r="S8" s="14"/>
     </row>
     <row r="9" spans="1:19" ht="45" x14ac:dyDescent="0.25">
-      <c r="A9" s="12">
+      <c r="A9" s="11">
         <v>2</v>
       </c>
-      <c r="B9" s="13" t="s">
+      <c r="B9" s="12" t="s">
         <v>182</v>
       </c>
-      <c r="C9" s="13" t="s">
+      <c r="C9" s="12" t="s">
         <v>183</v>
       </c>
-      <c r="D9" s="13" t="s">
+      <c r="D9" s="12" t="s">
         <v>184</v>
       </c>
-      <c r="E9" s="13" t="s">
+      <c r="E9" s="12" t="s">
         <v>182</v>
       </c>
-      <c r="F9" s="13" t="s">
+      <c r="F9" s="12" t="s">
         <v>182</v>
       </c>
-      <c r="G9" s="13" t="s">
+      <c r="G9" s="12" t="s">
         <v>185</v>
       </c>
-      <c r="H9" s="13" t="s">
+      <c r="H9" s="12" t="s">
         <v>186</v>
       </c>
-      <c r="I9" s="13" t="s">
+      <c r="I9" s="12" t="s">
         <v>186</v>
       </c>
-      <c r="J9" s="13" t="s">
+      <c r="J9" s="12" t="s">
         <v>23</v>
       </c>
-      <c r="K9" s="13" t="s">
+      <c r="K9" s="12" t="s">
         <v>187</v>
       </c>
-      <c r="L9" s="13" t="s">
+      <c r="L9" s="12" t="s">
         <v>25</v>
       </c>
-      <c r="M9" s="13" t="s">
+      <c r="M9" s="12" t="s">
         <v>188</v>
       </c>
-      <c r="N9" s="13" t="s">
+      <c r="N9" s="12" t="s">
         <v>36</v>
       </c>
-      <c r="O9" s="13" t="s">
+      <c r="O9" s="12" t="s">
         <v>189</v>
       </c>
-      <c r="P9" s="13" t="s">
-        <v>47</v>
-      </c>
-      <c r="Q9" s="15" t="s">
+      <c r="P9" s="12" t="s">
+        <v>47</v>
+      </c>
+      <c r="Q9" s="14" t="s">
         <v>351</v>
       </c>
       <c r="R9" s="7" t="s">
@@ -2107,51 +2113,51 @@
       </c>
     </row>
     <row r="10" spans="1:19" ht="45" x14ac:dyDescent="0.25">
-      <c r="A10" s="12">
+      <c r="A10" s="11">
         <v>8</v>
       </c>
-      <c r="B10" s="13" t="s">
+      <c r="B10" s="12" t="s">
         <v>290</v>
       </c>
-      <c r="C10" s="13" t="s">
+      <c r="C10" s="12" t="s">
         <v>291</v>
       </c>
-      <c r="D10" s="13" t="s">
+      <c r="D10" s="12" t="s">
         <v>184</v>
       </c>
-      <c r="E10" s="13" t="s">
+      <c r="E10" s="12" t="s">
         <v>292</v>
       </c>
-      <c r="F10" s="13" t="s">
+      <c r="F10" s="12" t="s">
         <v>290</v>
       </c>
-      <c r="G10" s="13" t="s">
+      <c r="G10" s="12" t="s">
         <v>293</v>
       </c>
-      <c r="H10" s="13" t="s">
+      <c r="H10" s="12" t="s">
         <v>294</v>
       </c>
-      <c r="I10" s="13" t="s">
+      <c r="I10" s="12" t="s">
         <v>295</v>
       </c>
-      <c r="J10" s="13" t="s">
+      <c r="J10" s="12" t="s">
         <v>23</v>
       </c>
-      <c r="K10" s="13" t="s">
+      <c r="K10" s="12" t="s">
         <v>296</v>
       </c>
-      <c r="L10" s="12"/>
-      <c r="M10" s="12"/>
-      <c r="N10" s="12"/>
-      <c r="O10" s="12"/>
-      <c r="P10" s="13" t="s">
-        <v>47</v>
-      </c>
-      <c r="Q10" s="14" t="s">
+      <c r="L10" s="11"/>
+      <c r="M10" s="11"/>
+      <c r="N10" s="11"/>
+      <c r="O10" s="11"/>
+      <c r="P10" s="12" t="s">
+        <v>47</v>
+      </c>
+      <c r="Q10" s="13" t="s">
         <v>330</v>
       </c>
-      <c r="R10" s="16"/>
-      <c r="S10" s="15"/>
+      <c r="R10" s="15"/>
+      <c r="S10" s="14"/>
     </row>
     <row r="11" spans="1:19" ht="45" x14ac:dyDescent="0.25">
       <c r="A11" s="3">
@@ -2299,51 +2305,51 @@
       </c>
     </row>
     <row r="14" spans="1:19" ht="60" x14ac:dyDescent="0.25">
-      <c r="A14" s="12">
+      <c r="A14" s="11">
         <v>8</v>
       </c>
-      <c r="B14" s="13" t="s">
+      <c r="B14" s="12" t="s">
         <v>282</v>
       </c>
-      <c r="C14" s="13" t="s">
+      <c r="C14" s="12" t="s">
         <v>283</v>
       </c>
-      <c r="D14" s="13" t="s">
+      <c r="D14" s="12" t="s">
         <v>284</v>
       </c>
-      <c r="E14" s="13" t="s">
+      <c r="E14" s="12" t="s">
         <v>285</v>
       </c>
-      <c r="F14" s="13" t="s">
+      <c r="F14" s="12" t="s">
         <v>282</v>
       </c>
-      <c r="G14" s="13" t="s">
+      <c r="G14" s="12" t="s">
         <v>286</v>
       </c>
-      <c r="H14" s="13" t="s">
+      <c r="H14" s="12" t="s">
         <v>287</v>
       </c>
-      <c r="I14" s="13" t="s">
+      <c r="I14" s="12" t="s">
         <v>288</v>
       </c>
-      <c r="J14" s="13" t="s">
+      <c r="J14" s="12" t="s">
         <v>25</v>
       </c>
-      <c r="K14" s="13" t="s">
+      <c r="K14" s="12" t="s">
         <v>289</v>
       </c>
-      <c r="L14" s="12"/>
-      <c r="M14" s="12"/>
-      <c r="N14" s="12"/>
-      <c r="O14" s="12"/>
-      <c r="P14" s="13" t="s">
-        <v>47</v>
-      </c>
-      <c r="Q14" s="14" t="s">
+      <c r="L14" s="11"/>
+      <c r="M14" s="11"/>
+      <c r="N14" s="11"/>
+      <c r="O14" s="11"/>
+      <c r="P14" s="12" t="s">
+        <v>47</v>
+      </c>
+      <c r="Q14" s="13" t="s">
         <v>333</v>
       </c>
-      <c r="R14" s="16"/>
-      <c r="S14" s="15"/>
+      <c r="R14" s="15"/>
+      <c r="S14" s="14"/>
     </row>
     <row r="15" spans="1:19" ht="45" x14ac:dyDescent="0.25">
       <c r="A15" s="3">
@@ -2439,102 +2445,102 @@
       </c>
     </row>
     <row r="17" spans="1:19" ht="210" x14ac:dyDescent="0.25">
-      <c r="A17" s="12">
+      <c r="A17" s="11">
         <v>40</v>
       </c>
-      <c r="B17" s="13" t="s">
+      <c r="B17" s="12" t="s">
         <v>312</v>
       </c>
-      <c r="C17" s="13" t="s">
+      <c r="C17" s="12" t="s">
         <v>313</v>
       </c>
-      <c r="D17" s="13" t="s">
+      <c r="D17" s="12" t="s">
         <v>50</v>
       </c>
-      <c r="E17" s="13" t="s">
+      <c r="E17" s="12" t="s">
         <v>314</v>
       </c>
-      <c r="F17" s="13" t="s">
+      <c r="F17" s="12" t="s">
         <v>312</v>
       </c>
-      <c r="G17" s="13" t="s">
+      <c r="G17" s="12" t="s">
         <v>315</v>
       </c>
-      <c r="H17" s="13" t="s">
+      <c r="H17" s="12" t="s">
         <v>316</v>
       </c>
-      <c r="I17" s="13" t="s">
+      <c r="I17" s="12" t="s">
         <v>317</v>
       </c>
-      <c r="J17" s="13" t="s">
+      <c r="J17" s="12" t="s">
         <v>25</v>
       </c>
-      <c r="K17" s="13" t="s">
+      <c r="K17" s="12" t="s">
         <v>318</v>
       </c>
-      <c r="L17" s="12"/>
-      <c r="M17" s="12"/>
-      <c r="N17" s="12"/>
-      <c r="O17" s="12"/>
-      <c r="P17" s="13" t="s">
-        <v>47</v>
-      </c>
-      <c r="Q17" s="14" t="s">
+      <c r="L17" s="11"/>
+      <c r="M17" s="11"/>
+      <c r="N17" s="11"/>
+      <c r="O17" s="11"/>
+      <c r="P17" s="12" t="s">
+        <v>47</v>
+      </c>
+      <c r="Q17" s="13" t="s">
         <v>337</v>
       </c>
-      <c r="R17" s="16" t="s">
+      <c r="R17" s="15" t="s">
         <v>338</v>
       </c>
-      <c r="S17" s="17" t="s">
+      <c r="S17" s="16" t="s">
         <v>352</v>
       </c>
     </row>
     <row r="18" spans="1:19" ht="90" x14ac:dyDescent="0.25">
-      <c r="A18" s="12">
+      <c r="A18" s="11">
         <v>12</v>
       </c>
-      <c r="B18" s="13" t="s">
+      <c r="B18" s="12" t="s">
         <v>308</v>
       </c>
-      <c r="C18" s="13" t="s">
+      <c r="C18" s="12" t="s">
         <v>309</v>
       </c>
-      <c r="D18" s="13" t="s">
+      <c r="D18" s="12" t="s">
         <v>41</v>
       </c>
-      <c r="E18" s="13" t="s">
+      <c r="E18" s="12" t="s">
         <v>310</v>
       </c>
-      <c r="F18" s="13" t="s">
+      <c r="F18" s="12" t="s">
         <v>308</v>
       </c>
-      <c r="G18" s="13" t="s">
+      <c r="G18" s="12" t="s">
         <v>52</v>
       </c>
-      <c r="H18" s="13" t="s">
+      <c r="H18" s="12" t="s">
         <v>53</v>
       </c>
-      <c r="I18" s="13" t="s">
+      <c r="I18" s="12" t="s">
         <v>54</v>
       </c>
-      <c r="J18" s="13" t="s">
+      <c r="J18" s="12" t="s">
         <v>23</v>
       </c>
-      <c r="K18" s="13" t="s">
+      <c r="K18" s="12" t="s">
         <v>311</v>
       </c>
-      <c r="L18" s="12"/>
-      <c r="M18" s="12"/>
-      <c r="N18" s="12"/>
-      <c r="O18" s="12"/>
-      <c r="P18" s="13" t="s">
-        <v>47</v>
-      </c>
-      <c r="Q18" s="15" t="s">
+      <c r="L18" s="11"/>
+      <c r="M18" s="11"/>
+      <c r="N18" s="11"/>
+      <c r="O18" s="11"/>
+      <c r="P18" s="12" t="s">
+        <v>47</v>
+      </c>
+      <c r="Q18" s="14" t="s">
         <v>340</v>
       </c>
-      <c r="R18" s="16"/>
-      <c r="S18" s="15"/>
+      <c r="R18" s="15"/>
+      <c r="S18" s="14"/>
     </row>
     <row r="19" spans="1:19" ht="30" x14ac:dyDescent="0.25">
       <c r="A19" s="3">
@@ -2582,53 +2588,53 @@
       </c>
     </row>
     <row r="20" spans="1:19" ht="45" x14ac:dyDescent="0.25">
-      <c r="A20" s="12">
+      <c r="A20" s="11">
         <v>1</v>
       </c>
-      <c r="B20" s="13" t="s">
+      <c r="B20" s="12" t="s">
         <v>48</v>
       </c>
-      <c r="C20" s="13" t="s">
+      <c r="C20" s="12" t="s">
         <v>49</v>
       </c>
-      <c r="D20" s="13" t="s">
+      <c r="D20" s="12" t="s">
         <v>50</v>
       </c>
-      <c r="E20" s="13" t="s">
+      <c r="E20" s="12" t="s">
         <v>51</v>
       </c>
-      <c r="F20" s="13" t="s">
+      <c r="F20" s="12" t="s">
         <v>48</v>
       </c>
-      <c r="G20" s="13" t="s">
+      <c r="G20" s="12" t="s">
         <v>52</v>
       </c>
-      <c r="H20" s="13" t="s">
+      <c r="H20" s="12" t="s">
         <v>53</v>
       </c>
-      <c r="I20" s="13" t="s">
+      <c r="I20" s="12" t="s">
         <v>54</v>
       </c>
-      <c r="J20" s="13" t="s">
+      <c r="J20" s="12" t="s">
         <v>23</v>
       </c>
-      <c r="K20" s="13" t="s">
+      <c r="K20" s="12" t="s">
         <v>55</v>
       </c>
-      <c r="L20" s="12"/>
-      <c r="M20" s="12"/>
-      <c r="N20" s="12"/>
-      <c r="O20" s="12"/>
-      <c r="P20" s="13" t="s">
-        <v>47</v>
-      </c>
-      <c r="Q20" s="15" t="s">
+      <c r="L20" s="11"/>
+      <c r="M20" s="11"/>
+      <c r="N20" s="11"/>
+      <c r="O20" s="11"/>
+      <c r="P20" s="12" t="s">
+        <v>47</v>
+      </c>
+      <c r="Q20" s="14" t="s">
         <v>336</v>
       </c>
-      <c r="R20" s="16" t="s">
+      <c r="R20" s="15" t="s">
         <v>335</v>
       </c>
-      <c r="S20" s="20" t="s">
+      <c r="S20" s="19" t="s">
         <v>355</v>
       </c>
     </row>
@@ -2678,112 +2684,112 @@
       </c>
     </row>
     <row r="22" spans="1:19" ht="45" x14ac:dyDescent="0.25">
-      <c r="A22" s="12">
+      <c r="A22" s="11">
         <v>2</v>
       </c>
-      <c r="B22" s="13" t="s">
+      <c r="B22" s="12" t="s">
         <v>174</v>
       </c>
-      <c r="C22" s="13" t="s">
+      <c r="C22" s="12" t="s">
         <v>175</v>
       </c>
-      <c r="D22" s="13" t="s">
+      <c r="D22" s="12" t="s">
         <v>76</v>
       </c>
-      <c r="E22" s="13" t="s">
+      <c r="E22" s="12" t="s">
         <v>174</v>
       </c>
-      <c r="F22" s="13" t="s">
+      <c r="F22" s="12" t="s">
         <v>174</v>
       </c>
-      <c r="G22" s="13" t="s">
+      <c r="G22" s="12" t="s">
         <v>176</v>
       </c>
-      <c r="H22" s="13" t="s">
+      <c r="H22" s="12" t="s">
         <v>177</v>
       </c>
-      <c r="I22" s="13" t="s">
+      <c r="I22" s="12" t="s">
         <v>178</v>
       </c>
-      <c r="J22" s="13" t="s">
+      <c r="J22" s="12" t="s">
         <v>25</v>
       </c>
-      <c r="K22" s="13" t="s">
+      <c r="K22" s="12" t="s">
         <v>179</v>
       </c>
-      <c r="L22" s="13" t="s">
+      <c r="L22" s="12" t="s">
         <v>23</v>
       </c>
-      <c r="M22" s="13" t="s">
+      <c r="M22" s="12" t="s">
         <v>180</v>
       </c>
-      <c r="N22" s="13" t="s">
+      <c r="N22" s="12" t="s">
         <v>36</v>
       </c>
-      <c r="O22" s="13" t="s">
+      <c r="O22" s="12" t="s">
         <v>181</v>
       </c>
-      <c r="P22" s="13" t="s">
-        <v>47</v>
-      </c>
-      <c r="Q22" s="15" t="s">
+      <c r="P22" s="12" t="s">
+        <v>47</v>
+      </c>
+      <c r="Q22" s="14" t="s">
         <v>341</v>
       </c>
-      <c r="R22" s="18" t="s">
+      <c r="R22" s="17" t="s">
         <v>353</v>
       </c>
-      <c r="S22" s="19" t="s">
+      <c r="S22" s="18" t="s">
         <v>354</v>
       </c>
     </row>
     <row r="23" spans="1:19" ht="45" x14ac:dyDescent="0.25">
-      <c r="A23" s="12">
+      <c r="A23" s="11">
         <v>1</v>
       </c>
-      <c r="B23" s="13" t="s">
+      <c r="B23" s="12" t="s">
         <v>126</v>
       </c>
-      <c r="C23" s="13" t="s">
+      <c r="C23" s="12" t="s">
         <v>127</v>
       </c>
-      <c r="D23" s="13" t="s">
+      <c r="D23" s="12" t="s">
         <v>128</v>
       </c>
-      <c r="E23" s="13" t="s">
+      <c r="E23" s="12" t="s">
         <v>129</v>
       </c>
-      <c r="F23" s="13" t="s">
+      <c r="F23" s="12" t="s">
         <v>126</v>
       </c>
-      <c r="G23" s="13" t="s">
+      <c r="G23" s="12" t="s">
         <v>130</v>
       </c>
-      <c r="H23" s="13" t="s">
+      <c r="H23" s="12" t="s">
         <v>131</v>
       </c>
-      <c r="I23" s="13" t="s">
+      <c r="I23" s="12" t="s">
         <v>132</v>
       </c>
-      <c r="J23" s="13" t="s">
+      <c r="J23" s="12" t="s">
         <v>36</v>
       </c>
-      <c r="K23" s="13" t="s">
+      <c r="K23" s="12" t="s">
         <v>133</v>
       </c>
-      <c r="L23" s="12"/>
-      <c r="M23" s="12"/>
-      <c r="N23" s="12"/>
-      <c r="O23" s="12"/>
-      <c r="P23" s="13" t="s">
-        <v>47</v>
-      </c>
-      <c r="Q23" s="15" t="s">
+      <c r="L23" s="11"/>
+      <c r="M23" s="11"/>
+      <c r="N23" s="11"/>
+      <c r="O23" s="11"/>
+      <c r="P23" s="12" t="s">
+        <v>47</v>
+      </c>
+      <c r="Q23" s="14" t="s">
         <v>343</v>
       </c>
       <c r="R23" s="7" t="s">
         <v>356</v>
       </c>
-      <c r="S23" s="20" t="s">
+      <c r="S23" s="19" t="s">
         <v>357</v>
       </c>
     </row>
@@ -2886,57 +2892,57 @@
       </c>
     </row>
     <row r="26" spans="1:19" ht="45" x14ac:dyDescent="0.25">
-      <c r="A26" s="12">
+      <c r="A26" s="11">
         <v>1</v>
       </c>
-      <c r="B26" s="13" t="s">
+      <c r="B26" s="12" t="s">
         <v>64</v>
       </c>
-      <c r="C26" s="13" t="s">
+      <c r="C26" s="12" t="s">
         <v>65</v>
       </c>
-      <c r="D26" s="13" t="s">
+      <c r="D26" s="12" t="s">
         <v>66</v>
       </c>
-      <c r="E26" s="13" t="s">
+      <c r="E26" s="12" t="s">
         <v>67</v>
       </c>
-      <c r="F26" s="13" t="s">
+      <c r="F26" s="12" t="s">
         <v>64</v>
       </c>
-      <c r="G26" s="13" t="s">
+      <c r="G26" s="12" t="s">
         <v>68</v>
       </c>
-      <c r="H26" s="13" t="s">
+      <c r="H26" s="12" t="s">
         <v>69</v>
       </c>
-      <c r="I26" s="13" t="s">
+      <c r="I26" s="12" t="s">
         <v>70</v>
       </c>
-      <c r="J26" s="13" t="s">
+      <c r="J26" s="12" t="s">
         <v>25</v>
       </c>
-      <c r="K26" s="13" t="s">
+      <c r="K26" s="12" t="s">
         <v>71</v>
       </c>
-      <c r="L26" s="13" t="s">
+      <c r="L26" s="12" t="s">
         <v>72</v>
       </c>
-      <c r="M26" s="13" t="s">
+      <c r="M26" s="12" t="s">
         <v>73</v>
       </c>
-      <c r="N26" s="12"/>
-      <c r="O26" s="12"/>
-      <c r="P26" s="13" t="s">
-        <v>47</v>
-      </c>
-      <c r="Q26" s="22" t="s">
+      <c r="N26" s="11"/>
+      <c r="O26" s="11"/>
+      <c r="P26" s="12" t="s">
+        <v>47</v>
+      </c>
+      <c r="Q26" s="21" t="s">
         <v>358</v>
       </c>
-      <c r="R26" s="16" t="s">
+      <c r="R26" s="15" t="s">
         <v>348</v>
       </c>
-      <c r="S26" s="24" t="s">
+      <c r="S26" s="23" t="s">
         <v>363</v>
       </c>
     </row>
@@ -2997,116 +3003,116 @@
       </c>
     </row>
     <row r="28" spans="1:19" ht="45" x14ac:dyDescent="0.25">
-      <c r="A28" s="12">
+      <c r="A28" s="11">
         <v>2</v>
       </c>
-      <c r="B28" s="13" t="s">
+      <c r="B28" s="12" t="s">
         <v>169</v>
       </c>
-      <c r="C28" s="13" t="s">
+      <c r="C28" s="12" t="s">
         <v>170</v>
       </c>
-      <c r="D28" s="13" t="s">
+      <c r="D28" s="12" t="s">
         <v>66</v>
       </c>
-      <c r="E28" s="13" t="s">
+      <c r="E28" s="12" t="s">
         <v>171</v>
       </c>
-      <c r="F28" s="13" t="s">
+      <c r="F28" s="12" t="s">
         <v>169</v>
       </c>
-      <c r="G28" s="13" t="s">
+      <c r="G28" s="12" t="s">
         <v>172</v>
       </c>
-      <c r="H28" s="13" t="s">
+      <c r="H28" s="12" t="s">
         <v>69</v>
       </c>
-      <c r="I28" s="13" t="s">
+      <c r="I28" s="12" t="s">
         <v>70</v>
       </c>
-      <c r="J28" s="13" t="s">
+      <c r="J28" s="12" t="s">
         <v>25</v>
       </c>
-      <c r="K28" s="13" t="s">
+      <c r="K28" s="12" t="s">
         <v>173</v>
       </c>
-      <c r="L28" s="12"/>
-      <c r="M28" s="12"/>
-      <c r="N28" s="12"/>
-      <c r="O28" s="12"/>
-      <c r="P28" s="13" t="s">
-        <v>47</v>
-      </c>
-      <c r="Q28" s="16" t="s">
+      <c r="L28" s="11"/>
+      <c r="M28" s="11"/>
+      <c r="N28" s="11"/>
+      <c r="O28" s="11"/>
+      <c r="P28" s="12" t="s">
+        <v>47</v>
+      </c>
+      <c r="Q28" s="15" t="s">
         <v>359</v>
       </c>
-      <c r="R28" s="16" t="s">
+      <c r="R28" s="15" t="s">
         <v>348</v>
       </c>
-      <c r="S28" s="17" t="s">
+      <c r="S28" s="16" t="s">
         <v>364</v>
       </c>
     </row>
     <row r="29" spans="1:19" ht="60" x14ac:dyDescent="0.25">
-      <c r="A29" s="12">
+      <c r="A29" s="11">
         <v>1</v>
       </c>
-      <c r="B29" s="13" t="s">
+      <c r="B29" s="12" t="s">
         <v>116</v>
       </c>
-      <c r="C29" s="13" t="s">
+      <c r="C29" s="12" t="s">
         <v>117</v>
       </c>
-      <c r="D29" s="13" t="s">
+      <c r="D29" s="12" t="s">
         <v>118</v>
       </c>
-      <c r="E29" s="13" t="s">
+      <c r="E29" s="12" t="s">
         <v>119</v>
       </c>
-      <c r="F29" s="13" t="s">
+      <c r="F29" s="12" t="s">
         <v>116</v>
       </c>
-      <c r="G29" s="13" t="s">
+      <c r="G29" s="12" t="s">
         <v>120</v>
       </c>
-      <c r="H29" s="13" t="s">
+      <c r="H29" s="12" t="s">
         <v>121</v>
       </c>
-      <c r="I29" s="13" t="s">
+      <c r="I29" s="12" t="s">
         <v>122</v>
       </c>
-      <c r="J29" s="13" t="s">
+      <c r="J29" s="12" t="s">
         <v>23</v>
       </c>
-      <c r="K29" s="13" t="s">
+      <c r="K29" s="12" t="s">
         <v>123</v>
       </c>
-      <c r="L29" s="13" t="s">
+      <c r="L29" s="12" t="s">
         <v>25</v>
       </c>
-      <c r="M29" s="13" t="s">
+      <c r="M29" s="12" t="s">
         <v>124</v>
       </c>
-      <c r="N29" s="13" t="s">
+      <c r="N29" s="12" t="s">
         <v>36</v>
       </c>
-      <c r="O29" s="13" t="s">
+      <c r="O29" s="12" t="s">
         <v>125</v>
       </c>
-      <c r="P29" s="13" t="s">
-        <v>47</v>
-      </c>
-      <c r="Q29" s="22" t="s">
+      <c r="P29" s="12" t="s">
+        <v>47</v>
+      </c>
+      <c r="Q29" s="21" t="s">
         <v>323</v>
       </c>
-      <c r="R29" s="16"/>
-      <c r="S29" s="15"/>
+      <c r="R29" s="15"/>
+      <c r="S29" s="14"/>
     </row>
     <row r="30" spans="1:19" ht="45" x14ac:dyDescent="0.25">
       <c r="A30" s="3">
         <v>5</v>
       </c>
-      <c r="B30" s="4" t="s">
+      <c r="B30" s="26" t="s">
         <v>268</v>
       </c>
       <c r="C30" s="4" t="s">
@@ -3152,692 +3158,696 @@
       </c>
     </row>
     <row r="31" spans="1:19" ht="60" x14ac:dyDescent="0.25">
-      <c r="A31" s="12">
+      <c r="A31" s="11">
         <v>5</v>
       </c>
-      <c r="B31" s="13" t="s">
+      <c r="B31" s="12" t="s">
         <v>247</v>
       </c>
-      <c r="C31" s="13" t="s">
+      <c r="C31" s="12" t="s">
         <v>248</v>
       </c>
-      <c r="D31" s="13" t="s">
+      <c r="D31" s="12" t="s">
         <v>249</v>
       </c>
-      <c r="E31" s="13" t="s">
+      <c r="E31" s="12" t="s">
         <v>247</v>
       </c>
-      <c r="F31" s="13" t="s">
+      <c r="F31" s="12" t="s">
         <v>247</v>
       </c>
-      <c r="G31" s="13" t="s">
+      <c r="G31" s="12" t="s">
         <v>250</v>
       </c>
-      <c r="H31" s="13" t="s">
+      <c r="H31" s="12" t="s">
         <v>251</v>
       </c>
-      <c r="I31" s="13" t="s">
+      <c r="I31" s="12" t="s">
         <v>252</v>
       </c>
-      <c r="J31" s="13" t="s">
+      <c r="J31" s="12" t="s">
         <v>36</v>
       </c>
-      <c r="K31" s="13" t="s">
+      <c r="K31" s="12" t="s">
         <v>253</v>
       </c>
-      <c r="L31" s="13" t="s">
+      <c r="L31" s="12" t="s">
         <v>25</v>
       </c>
-      <c r="M31" s="13" t="s">
+      <c r="M31" s="12" t="s">
         <v>254</v>
       </c>
-      <c r="N31" s="13" t="s">
+      <c r="N31" s="12" t="s">
         <v>23</v>
       </c>
-      <c r="O31" s="13" t="s">
+      <c r="O31" s="12" t="s">
         <v>255</v>
       </c>
-      <c r="P31" s="13" t="s">
-        <v>47</v>
-      </c>
-      <c r="Q31" s="14" t="s">
+      <c r="P31" s="12" t="s">
+        <v>47</v>
+      </c>
+      <c r="Q31" s="13" t="s">
         <v>347</v>
       </c>
-      <c r="R31" s="21" t="s">
+      <c r="R31" s="20" t="s">
         <v>342</v>
       </c>
     </row>
     <row r="32" spans="1:19" ht="45" x14ac:dyDescent="0.25">
-      <c r="A32" s="12">
+      <c r="A32" s="11">
         <v>2</v>
       </c>
-      <c r="B32" s="13" t="s">
+      <c r="B32" s="12" t="s">
         <v>196</v>
       </c>
-      <c r="C32" s="13" t="s">
+      <c r="C32" s="12" t="s">
         <v>197</v>
       </c>
-      <c r="D32" s="13" t="s">
+      <c r="D32" s="12" t="s">
         <v>198</v>
       </c>
-      <c r="E32" s="13" t="s">
+      <c r="E32" s="12" t="s">
         <v>199</v>
       </c>
-      <c r="F32" s="13" t="s">
+      <c r="F32" s="12" t="s">
         <v>196</v>
       </c>
-      <c r="G32" s="13" t="s">
+      <c r="G32" s="12" t="s">
         <v>200</v>
       </c>
-      <c r="H32" s="13" t="s">
+      <c r="H32" s="12" t="s">
         <v>201</v>
       </c>
-      <c r="I32" s="13" t="s">
+      <c r="I32" s="12" t="s">
         <v>70</v>
       </c>
-      <c r="J32" s="13" t="s">
+      <c r="J32" s="12" t="s">
         <v>23</v>
       </c>
-      <c r="K32" s="13" t="s">
+      <c r="K32" s="12" t="s">
         <v>202</v>
       </c>
-      <c r="L32" s="13" t="s">
+      <c r="L32" s="12" t="s">
         <v>25</v>
       </c>
-      <c r="M32" s="13" t="s">
+      <c r="M32" s="12" t="s">
         <v>203</v>
       </c>
-      <c r="N32" s="13" t="s">
+      <c r="N32" s="12" t="s">
         <v>36</v>
       </c>
-      <c r="O32" s="13" t="s">
+      <c r="O32" s="12" t="s">
         <v>204</v>
       </c>
-      <c r="P32" s="13" t="s">
-        <v>47</v>
-      </c>
-      <c r="Q32" s="26" t="s">
+      <c r="P32" s="12" t="s">
+        <v>47</v>
+      </c>
+      <c r="Q32" s="25" t="s">
         <v>334</v>
       </c>
-      <c r="R32" s="16"/>
-      <c r="S32" s="15"/>
+      <c r="R32" s="15"/>
+      <c r="S32" s="14"/>
     </row>
     <row r="33" spans="1:19" ht="45" x14ac:dyDescent="0.25">
-      <c r="A33" s="3">
+      <c r="A33" s="11">
         <v>4</v>
       </c>
-      <c r="B33" s="4" t="s">
+      <c r="B33" s="12" t="s">
         <v>235</v>
       </c>
-      <c r="C33" s="4" t="s">
+      <c r="C33" s="12" t="s">
         <v>236</v>
       </c>
-      <c r="D33" s="4" t="s">
+      <c r="D33" s="12" t="s">
         <v>58</v>
       </c>
-      <c r="E33" s="4" t="s">
+      <c r="E33" s="12" t="s">
         <v>235</v>
       </c>
-      <c r="F33" s="4" t="s">
+      <c r="F33" s="12" t="s">
         <v>235</v>
       </c>
-      <c r="G33" s="4" t="s">
+      <c r="G33" s="12" t="s">
         <v>237</v>
       </c>
-      <c r="H33" s="4" t="s">
+      <c r="H33" s="12" t="s">
         <v>238</v>
       </c>
-      <c r="I33" s="3"/>
-      <c r="J33" s="4" t="s">
+      <c r="I33" s="11"/>
+      <c r="J33" s="12" t="s">
         <v>25</v>
       </c>
-      <c r="K33" s="4" t="s">
+      <c r="K33" s="12" t="s">
         <v>239</v>
       </c>
-      <c r="L33" s="4" t="s">
+      <c r="L33" s="12" t="s">
         <v>36</v>
       </c>
-      <c r="M33" s="4" t="s">
+      <c r="M33" s="12" t="s">
         <v>240</v>
       </c>
-      <c r="N33" s="3"/>
-      <c r="O33" s="3"/>
-      <c r="P33" s="4" t="s">
-        <v>47</v>
-      </c>
-      <c r="Q33" s="11" t="s">
+      <c r="N33" s="11"/>
+      <c r="O33" s="11"/>
+      <c r="P33" s="12" t="s">
+        <v>47</v>
+      </c>
+      <c r="Q33" s="25" t="s">
         <v>334</v>
       </c>
+      <c r="R33" s="15"/>
+      <c r="S33" s="14"/>
     </row>
     <row r="34" spans="1:19" ht="30" x14ac:dyDescent="0.25">
-      <c r="A34" s="3">
+      <c r="A34" s="11">
         <v>4</v>
       </c>
-      <c r="B34" s="4" t="s">
+      <c r="B34" s="12" t="s">
         <v>241</v>
       </c>
-      <c r="C34" s="4" t="s">
+      <c r="C34" s="12" t="s">
         <v>242</v>
       </c>
-      <c r="D34" s="4" t="s">
+      <c r="D34" s="12" t="s">
         <v>118</v>
       </c>
-      <c r="E34" s="4" t="s">
+      <c r="E34" s="12" t="s">
         <v>241</v>
       </c>
-      <c r="F34" s="4" t="s">
+      <c r="F34" s="12" t="s">
         <v>241</v>
       </c>
-      <c r="G34" s="4" t="s">
+      <c r="G34" s="12" t="s">
         <v>243</v>
       </c>
-      <c r="H34" s="4" t="s">
+      <c r="H34" s="12" t="s">
         <v>244</v>
       </c>
-      <c r="I34" s="4" t="s">
+      <c r="I34" s="12" t="s">
         <v>245</v>
       </c>
-      <c r="J34" s="4" t="s">
+      <c r="J34" s="12" t="s">
         <v>23</v>
       </c>
-      <c r="K34" s="4" t="s">
+      <c r="K34" s="12" t="s">
         <v>246</v>
       </c>
-      <c r="L34" s="3"/>
-      <c r="M34" s="3"/>
-      <c r="N34" s="3"/>
-      <c r="O34" s="3"/>
-      <c r="P34" s="4" t="s">
-        <v>47</v>
-      </c>
-      <c r="Q34" s="11" t="s">
+      <c r="L34" s="11"/>
+      <c r="M34" s="11"/>
+      <c r="N34" s="11"/>
+      <c r="O34" s="11"/>
+      <c r="P34" s="12" t="s">
+        <v>47</v>
+      </c>
+      <c r="Q34" s="25" t="s">
         <v>334</v>
       </c>
+      <c r="R34" s="15"/>
+      <c r="S34" s="14"/>
     </row>
     <row r="35" spans="1:19" ht="30" x14ac:dyDescent="0.25">
-      <c r="A35" s="12">
+      <c r="A35" s="11">
         <v>1</v>
       </c>
-      <c r="B35" s="13" t="s">
+      <c r="B35" s="12" t="s">
         <v>102</v>
       </c>
-      <c r="C35" s="13" t="s">
+      <c r="C35" s="12" t="s">
         <v>103</v>
       </c>
-      <c r="D35" s="13" t="s">
+      <c r="D35" s="12" t="s">
         <v>86</v>
       </c>
-      <c r="E35" s="13" t="s">
+      <c r="E35" s="12" t="s">
         <v>102</v>
       </c>
-      <c r="F35" s="13" t="s">
+      <c r="F35" s="12" t="s">
         <v>102</v>
       </c>
-      <c r="G35" s="13" t="s">
+      <c r="G35" s="12" t="s">
         <v>87</v>
       </c>
-      <c r="H35" s="13" t="s">
+      <c r="H35" s="12" t="s">
         <v>102</v>
       </c>
-      <c r="I35" s="12"/>
-      <c r="J35" s="13" t="s">
+      <c r="I35" s="11"/>
+      <c r="J35" s="12" t="s">
         <v>25</v>
       </c>
-      <c r="K35" s="13" t="s">
+      <c r="K35" s="12" t="s">
         <v>104</v>
       </c>
-      <c r="L35" s="13" t="s">
+      <c r="L35" s="12" t="s">
         <v>36</v>
       </c>
-      <c r="M35" s="13" t="s">
+      <c r="M35" s="12" t="s">
         <v>105</v>
       </c>
-      <c r="N35" s="12"/>
-      <c r="O35" s="12"/>
-      <c r="P35" s="13" t="s">
-        <v>47</v>
-      </c>
-      <c r="Q35" s="22" t="s">
+      <c r="N35" s="11"/>
+      <c r="O35" s="11"/>
+      <c r="P35" s="12" t="s">
+        <v>47</v>
+      </c>
+      <c r="Q35" s="21" t="s">
         <v>323</v>
       </c>
-      <c r="R35" s="16"/>
-      <c r="S35" s="15"/>
+      <c r="R35" s="15"/>
+      <c r="S35" s="14"/>
     </row>
     <row r="36" spans="1:19" ht="45" x14ac:dyDescent="0.25">
-      <c r="A36" s="12">
+      <c r="A36" s="11">
         <v>1</v>
       </c>
-      <c r="B36" s="13" t="s">
+      <c r="B36" s="12" t="s">
         <v>91</v>
       </c>
-      <c r="C36" s="13" t="s">
+      <c r="C36" s="12" t="s">
         <v>92</v>
       </c>
-      <c r="D36" s="13" t="s">
+      <c r="D36" s="12" t="s">
         <v>86</v>
       </c>
-      <c r="E36" s="13" t="s">
+      <c r="E36" s="12" t="s">
         <v>91</v>
       </c>
-      <c r="F36" s="13" t="s">
+      <c r="F36" s="12" t="s">
         <v>91</v>
       </c>
-      <c r="G36" s="13" t="s">
+      <c r="G36" s="12" t="s">
         <v>93</v>
       </c>
-      <c r="H36" s="13" t="s">
+      <c r="H36" s="12" t="s">
         <v>91</v>
       </c>
-      <c r="I36" s="12"/>
-      <c r="J36" s="13" t="s">
+      <c r="I36" s="11"/>
+      <c r="J36" s="12" t="s">
         <v>23</v>
       </c>
-      <c r="K36" s="13" t="s">
+      <c r="K36" s="12" t="s">
         <v>94</v>
       </c>
-      <c r="L36" s="13" t="s">
+      <c r="L36" s="12" t="s">
         <v>25</v>
       </c>
-      <c r="M36" s="13" t="s">
+      <c r="M36" s="12" t="s">
         <v>95</v>
       </c>
-      <c r="N36" s="13" t="s">
+      <c r="N36" s="12" t="s">
         <v>36</v>
       </c>
-      <c r="O36" s="13" t="s">
+      <c r="O36" s="12" t="s">
         <v>96</v>
       </c>
-      <c r="P36" s="13" t="s">
-        <v>47</v>
-      </c>
-      <c r="Q36" s="22" t="s">
+      <c r="P36" s="12" t="s">
+        <v>47</v>
+      </c>
+      <c r="Q36" s="21" t="s">
         <v>323</v>
       </c>
-      <c r="R36" s="16"/>
-      <c r="S36" s="24" t="s">
+      <c r="R36" s="15"/>
+      <c r="S36" s="23" t="s">
         <v>360</v>
       </c>
     </row>
     <row r="37" spans="1:19" ht="45" x14ac:dyDescent="0.25">
-      <c r="A37" s="12">
+      <c r="A37" s="11">
         <v>1</v>
       </c>
-      <c r="B37" s="13" t="s">
+      <c r="B37" s="12" t="s">
         <v>106</v>
       </c>
-      <c r="C37" s="13" t="s">
+      <c r="C37" s="12" t="s">
         <v>107</v>
       </c>
-      <c r="D37" s="13" t="s">
+      <c r="D37" s="12" t="s">
         <v>86</v>
       </c>
-      <c r="E37" s="13" t="s">
+      <c r="E37" s="12" t="s">
         <v>106</v>
       </c>
-      <c r="F37" s="13" t="s">
+      <c r="F37" s="12" t="s">
         <v>106</v>
       </c>
-      <c r="G37" s="13" t="s">
+      <c r="G37" s="12" t="s">
         <v>93</v>
       </c>
-      <c r="H37" s="13" t="s">
+      <c r="H37" s="12" t="s">
         <v>106</v>
       </c>
-      <c r="I37" s="12"/>
-      <c r="J37" s="13" t="s">
+      <c r="I37" s="11"/>
+      <c r="J37" s="12" t="s">
         <v>23</v>
       </c>
-      <c r="K37" s="13" t="s">
+      <c r="K37" s="12" t="s">
         <v>108</v>
       </c>
-      <c r="L37" s="13" t="s">
+      <c r="L37" s="12" t="s">
         <v>25</v>
       </c>
-      <c r="M37" s="13" t="s">
+      <c r="M37" s="12" t="s">
         <v>109</v>
       </c>
-      <c r="N37" s="13" t="s">
+      <c r="N37" s="12" t="s">
         <v>36</v>
       </c>
-      <c r="O37" s="13" t="s">
+      <c r="O37" s="12" t="s">
         <v>110</v>
       </c>
-      <c r="P37" s="13" t="s">
-        <v>47</v>
-      </c>
-      <c r="Q37" s="22" t="s">
+      <c r="P37" s="12" t="s">
+        <v>47</v>
+      </c>
+      <c r="Q37" s="21" t="s">
         <v>323</v>
       </c>
-      <c r="R37" s="16"/>
-      <c r="S37" s="24" t="s">
+      <c r="R37" s="15"/>
+      <c r="S37" s="23" t="s">
         <v>360</v>
       </c>
     </row>
     <row r="38" spans="1:19" ht="45" x14ac:dyDescent="0.25">
-      <c r="A38" s="12">
+      <c r="A38" s="11">
         <v>1</v>
       </c>
-      <c r="B38" s="13" t="s">
+      <c r="B38" s="12" t="s">
         <v>97</v>
       </c>
-      <c r="C38" s="13" t="s">
+      <c r="C38" s="12" t="s">
         <v>98</v>
       </c>
-      <c r="D38" s="13" t="s">
+      <c r="D38" s="12" t="s">
         <v>86</v>
       </c>
-      <c r="E38" s="13" t="s">
+      <c r="E38" s="12" t="s">
         <v>97</v>
       </c>
-      <c r="F38" s="13" t="s">
+      <c r="F38" s="12" t="s">
         <v>97</v>
       </c>
-      <c r="G38" s="13" t="s">
+      <c r="G38" s="12" t="s">
         <v>93</v>
       </c>
-      <c r="H38" s="13" t="s">
+      <c r="H38" s="12" t="s">
         <v>97</v>
       </c>
-      <c r="I38" s="12"/>
-      <c r="J38" s="13" t="s">
+      <c r="I38" s="11"/>
+      <c r="J38" s="12" t="s">
         <v>23</v>
       </c>
-      <c r="K38" s="13" t="s">
+      <c r="K38" s="12" t="s">
         <v>99</v>
       </c>
-      <c r="L38" s="13" t="s">
+      <c r="L38" s="12" t="s">
         <v>25</v>
       </c>
-      <c r="M38" s="13" t="s">
+      <c r="M38" s="12" t="s">
         <v>100</v>
       </c>
-      <c r="N38" s="13" t="s">
+      <c r="N38" s="12" t="s">
         <v>36</v>
       </c>
-      <c r="O38" s="13" t="s">
+      <c r="O38" s="12" t="s">
         <v>101</v>
       </c>
-      <c r="P38" s="13" t="s">
-        <v>47</v>
-      </c>
-      <c r="Q38" s="22" t="s">
+      <c r="P38" s="12" t="s">
+        <v>47</v>
+      </c>
+      <c r="Q38" s="21" t="s">
         <v>323</v>
       </c>
-      <c r="R38" s="16"/>
-      <c r="S38" s="24" t="s">
+      <c r="R38" s="15"/>
+      <c r="S38" s="23" t="s">
         <v>360</v>
       </c>
     </row>
     <row r="39" spans="1:19" ht="45" x14ac:dyDescent="0.25">
-      <c r="A39" s="12">
+      <c r="A39" s="11">
         <v>1</v>
       </c>
-      <c r="B39" s="13" t="s">
+      <c r="B39" s="12" t="s">
         <v>84</v>
       </c>
-      <c r="C39" s="13" t="s">
+      <c r="C39" s="12" t="s">
         <v>85</v>
       </c>
-      <c r="D39" s="13" t="s">
+      <c r="D39" s="12" t="s">
         <v>86</v>
       </c>
-      <c r="E39" s="13" t="s">
+      <c r="E39" s="12" t="s">
         <v>84</v>
       </c>
-      <c r="F39" s="13" t="s">
+      <c r="F39" s="12" t="s">
         <v>84</v>
       </c>
-      <c r="G39" s="13" t="s">
+      <c r="G39" s="12" t="s">
         <v>87</v>
       </c>
-      <c r="H39" s="13" t="s">
+      <c r="H39" s="12" t="s">
         <v>84</v>
       </c>
-      <c r="I39" s="12"/>
-      <c r="J39" s="13" t="s">
+      <c r="I39" s="11"/>
+      <c r="J39" s="12" t="s">
         <v>23</v>
       </c>
-      <c r="K39" s="13" t="s">
+      <c r="K39" s="12" t="s">
         <v>88</v>
       </c>
-      <c r="L39" s="13" t="s">
+      <c r="L39" s="12" t="s">
         <v>25</v>
       </c>
-      <c r="M39" s="13" t="s">
+      <c r="M39" s="12" t="s">
         <v>89</v>
       </c>
-      <c r="N39" s="13" t="s">
+      <c r="N39" s="12" t="s">
         <v>36</v>
       </c>
-      <c r="O39" s="13" t="s">
+      <c r="O39" s="12" t="s">
         <v>90</v>
       </c>
-      <c r="P39" s="13" t="s">
-        <v>47</v>
-      </c>
-      <c r="Q39" s="22" t="s">
+      <c r="P39" s="12" t="s">
+        <v>47</v>
+      </c>
+      <c r="Q39" s="21" t="s">
         <v>323</v>
       </c>
-      <c r="R39" s="16"/>
-      <c r="S39" s="24" t="s">
+      <c r="R39" s="15"/>
+      <c r="S39" s="23" t="s">
         <v>360</v>
       </c>
     </row>
     <row r="40" spans="1:19" ht="45" x14ac:dyDescent="0.25">
-      <c r="A40" s="12">
+      <c r="A40" s="11">
         <v>1</v>
       </c>
-      <c r="B40" s="13" t="s">
+      <c r="B40" s="12" t="s">
         <v>111</v>
       </c>
-      <c r="C40" s="13" t="s">
+      <c r="C40" s="12" t="s">
         <v>112</v>
       </c>
-      <c r="D40" s="13" t="s">
+      <c r="D40" s="12" t="s">
         <v>86</v>
       </c>
-      <c r="E40" s="13" t="s">
+      <c r="E40" s="12" t="s">
         <v>111</v>
       </c>
-      <c r="F40" s="13" t="s">
+      <c r="F40" s="12" t="s">
         <v>111</v>
       </c>
-      <c r="G40" s="13" t="s">
+      <c r="G40" s="12" t="s">
         <v>93</v>
       </c>
-      <c r="H40" s="13" t="s">
+      <c r="H40" s="12" t="s">
         <v>111</v>
       </c>
-      <c r="I40" s="12"/>
-      <c r="J40" s="13" t="s">
+      <c r="I40" s="11"/>
+      <c r="J40" s="12" t="s">
         <v>23</v>
       </c>
-      <c r="K40" s="13" t="s">
+      <c r="K40" s="12" t="s">
         <v>113</v>
       </c>
-      <c r="L40" s="13" t="s">
+      <c r="L40" s="12" t="s">
         <v>25</v>
       </c>
-      <c r="M40" s="13" t="s">
+      <c r="M40" s="12" t="s">
         <v>114</v>
       </c>
-      <c r="N40" s="13" t="s">
+      <c r="N40" s="12" t="s">
         <v>36</v>
       </c>
-      <c r="O40" s="13" t="s">
+      <c r="O40" s="12" t="s">
         <v>115</v>
       </c>
-      <c r="P40" s="13" t="s">
-        <v>47</v>
-      </c>
-      <c r="Q40" s="22" t="s">
+      <c r="P40" s="12" t="s">
+        <v>47</v>
+      </c>
+      <c r="Q40" s="21" t="s">
         <v>323</v>
       </c>
-      <c r="R40" s="16"/>
-      <c r="S40" s="15"/>
+      <c r="R40" s="15"/>
+      <c r="S40" s="14"/>
     </row>
     <row r="41" spans="1:19" ht="45" x14ac:dyDescent="0.25">
-      <c r="A41" s="12">
+      <c r="A41" s="11">
         <v>1</v>
       </c>
-      <c r="B41" s="13" t="s">
+      <c r="B41" s="12" t="s">
         <v>56</v>
       </c>
-      <c r="C41" s="13" t="s">
+      <c r="C41" s="12" t="s">
         <v>57</v>
       </c>
-      <c r="D41" s="13" t="s">
+      <c r="D41" s="12" t="s">
         <v>58</v>
       </c>
-      <c r="E41" s="13" t="s">
+      <c r="E41" s="12" t="s">
         <v>56</v>
       </c>
-      <c r="F41" s="13" t="s">
+      <c r="F41" s="12" t="s">
         <v>56</v>
       </c>
-      <c r="G41" s="13" t="s">
+      <c r="G41" s="12" t="s">
         <v>59</v>
       </c>
-      <c r="H41" s="13" t="s">
+      <c r="H41" s="12" t="s">
         <v>56</v>
       </c>
-      <c r="I41" s="13" t="s">
+      <c r="I41" s="12" t="s">
         <v>60</v>
       </c>
-      <c r="J41" s="13" t="s">
+      <c r="J41" s="12" t="s">
         <v>23</v>
       </c>
-      <c r="K41" s="13" t="s">
+      <c r="K41" s="12" t="s">
         <v>61</v>
       </c>
-      <c r="L41" s="13" t="s">
+      <c r="L41" s="12" t="s">
         <v>25</v>
       </c>
-      <c r="M41" s="13" t="s">
+      <c r="M41" s="12" t="s">
         <v>62</v>
       </c>
-      <c r="N41" s="13" t="s">
+      <c r="N41" s="12" t="s">
         <v>36</v>
       </c>
-      <c r="O41" s="13" t="s">
+      <c r="O41" s="12" t="s">
         <v>63</v>
       </c>
-      <c r="P41" s="13" t="s">
-        <v>47</v>
-      </c>
-      <c r="Q41" s="22" t="s">
+      <c r="P41" s="12" t="s">
+        <v>47</v>
+      </c>
+      <c r="Q41" s="21" t="s">
         <v>325</v>
       </c>
-      <c r="R41" s="16"/>
-      <c r="S41" s="15"/>
+      <c r="R41" s="15"/>
+      <c r="S41" s="14"/>
     </row>
     <row r="42" spans="1:19" ht="60" x14ac:dyDescent="0.25">
-      <c r="A42" s="12">
+      <c r="A42" s="11">
         <v>3</v>
       </c>
-      <c r="B42" s="13" t="s">
+      <c r="B42" s="12" t="s">
         <v>217</v>
       </c>
-      <c r="C42" s="13" t="s">
+      <c r="C42" s="12" t="s">
         <v>218</v>
       </c>
-      <c r="D42" s="13" t="s">
+      <c r="D42" s="12" t="s">
         <v>86</v>
       </c>
-      <c r="E42" s="13" t="s">
+      <c r="E42" s="12" t="s">
         <v>217</v>
       </c>
-      <c r="F42" s="13" t="s">
+      <c r="F42" s="12" t="s">
         <v>217</v>
       </c>
-      <c r="G42" s="13" t="s">
+      <c r="G42" s="12" t="s">
         <v>219</v>
       </c>
-      <c r="H42" s="13" t="s">
+      <c r="H42" s="12" t="s">
         <v>220</v>
       </c>
-      <c r="I42" s="12"/>
-      <c r="J42" s="13" t="s">
+      <c r="I42" s="11"/>
+      <c r="J42" s="12" t="s">
         <v>23</v>
       </c>
-      <c r="K42" s="13" t="s">
+      <c r="K42" s="12" t="s">
         <v>221</v>
       </c>
-      <c r="L42" s="13" t="s">
+      <c r="L42" s="12" t="s">
         <v>25</v>
       </c>
-      <c r="M42" s="13" t="s">
+      <c r="M42" s="12" t="s">
         <v>222</v>
       </c>
-      <c r="N42" s="13" t="s">
+      <c r="N42" s="12" t="s">
         <v>36</v>
       </c>
-      <c r="O42" s="13" t="s">
+      <c r="O42" s="12" t="s">
         <v>223</v>
       </c>
-      <c r="P42" s="13" t="s">
-        <v>47</v>
-      </c>
-      <c r="Q42" s="22" t="s">
+      <c r="P42" s="12" t="s">
+        <v>47</v>
+      </c>
+      <c r="Q42" s="21" t="s">
         <v>323</v>
       </c>
-      <c r="R42" s="16"/>
-      <c r="S42" s="25" t="s">
+      <c r="R42" s="15"/>
+      <c r="S42" s="24" t="s">
         <v>361</v>
       </c>
     </row>
     <row r="43" spans="1:19" ht="60" x14ac:dyDescent="0.25">
-      <c r="A43" s="12">
+      <c r="A43" s="11">
         <v>5</v>
       </c>
-      <c r="B43" s="13" t="s">
+      <c r="B43" s="12" t="s">
         <v>262</v>
       </c>
-      <c r="C43" s="13" t="s">
+      <c r="C43" s="12" t="s">
         <v>263</v>
       </c>
-      <c r="D43" s="13" t="s">
+      <c r="D43" s="12" t="s">
         <v>86</v>
       </c>
-      <c r="E43" s="13" t="s">
+      <c r="E43" s="12" t="s">
         <v>262</v>
       </c>
-      <c r="F43" s="13" t="s">
+      <c r="F43" s="12" t="s">
         <v>262</v>
       </c>
-      <c r="G43" s="13" t="s">
+      <c r="G43" s="12" t="s">
         <v>219</v>
       </c>
-      <c r="H43" s="13" t="s">
+      <c r="H43" s="12" t="s">
         <v>264</v>
       </c>
-      <c r="I43" s="12"/>
-      <c r="J43" s="13" t="s">
+      <c r="I43" s="11"/>
+      <c r="J43" s="12" t="s">
         <v>23</v>
       </c>
-      <c r="K43" s="13" t="s">
+      <c r="K43" s="12" t="s">
         <v>265</v>
       </c>
-      <c r="L43" s="13" t="s">
+      <c r="L43" s="12" t="s">
         <v>25</v>
       </c>
-      <c r="M43" s="13" t="s">
+      <c r="M43" s="12" t="s">
         <v>266</v>
       </c>
-      <c r="N43" s="13" t="s">
+      <c r="N43" s="12" t="s">
         <v>36</v>
       </c>
-      <c r="O43" s="13" t="s">
+      <c r="O43" s="12" t="s">
         <v>267</v>
       </c>
-      <c r="P43" s="13" t="s">
-        <v>47</v>
-      </c>
-      <c r="Q43" s="22" t="s">
+      <c r="P43" s="12" t="s">
+        <v>47</v>
+      </c>
+      <c r="Q43" s="21" t="s">
         <v>323</v>
       </c>
-      <c r="R43" s="16"/>
-      <c r="S43" s="25" t="s">
+      <c r="R43" s="15"/>
+      <c r="S43" s="24" t="s">
         <v>362</v>
       </c>
     </row>

</xml_diff>

<commit_message>
changed NLV74HC32ADTR2G (U15,U16) to 30783 out of TE.DbLib/LOGIC
</commit_message>
<xml_diff>
--- a/Using Trenz Library/BOM_MissingComponents_in_process_Simon.xlsx
+++ b/Using Trenz Library/BOM_MissingComponents_in_process_Simon.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="646" uniqueCount="365">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="647" uniqueCount="366">
   <si>
     <t>Quantity</t>
   </si>
@@ -1122,6 +1122,9 @@
   </si>
   <si>
     <t>used ISO7742QDWRQ1</t>
+  </si>
+  <si>
+    <t>used NLV74HC32ADTR2G</t>
   </si>
 </sst>
 </file>
@@ -2843,52 +2846,56 @@
       </c>
     </row>
     <row r="25" spans="1:19" ht="60" x14ac:dyDescent="0.25">
-      <c r="A25" s="3">
+      <c r="A25" s="11">
         <v>2</v>
       </c>
-      <c r="B25" s="4" t="s">
+      <c r="B25" s="12" t="s">
         <v>28</v>
       </c>
-      <c r="C25" s="4" t="s">
+      <c r="C25" s="12" t="s">
         <v>29</v>
       </c>
-      <c r="D25" s="4" t="s">
+      <c r="D25" s="12" t="s">
         <v>30</v>
       </c>
-      <c r="E25" s="4" t="s">
+      <c r="E25" s="12" t="s">
         <v>31</v>
       </c>
-      <c r="F25" s="4" t="s">
+      <c r="F25" s="12" t="s">
         <v>28</v>
       </c>
-      <c r="G25" s="4" t="s">
+      <c r="G25" s="12" t="s">
         <v>32</v>
       </c>
-      <c r="H25" s="4" t="s">
+      <c r="H25" s="12" t="s">
         <v>33</v>
       </c>
-      <c r="I25" s="4" t="s">
+      <c r="I25" s="12" t="s">
         <v>34</v>
       </c>
-      <c r="J25" s="4" t="s">
+      <c r="J25" s="12" t="s">
         <v>25</v>
       </c>
-      <c r="K25" s="4" t="s">
+      <c r="K25" s="12" t="s">
         <v>35</v>
       </c>
-      <c r="L25" s="4" t="s">
+      <c r="L25" s="12" t="s">
         <v>36</v>
       </c>
-      <c r="M25" s="4" t="s">
+      <c r="M25" s="12" t="s">
         <v>37</v>
       </c>
-      <c r="N25" s="3"/>
-      <c r="O25" s="3"/>
-      <c r="P25" s="4" t="s">
+      <c r="N25" s="11"/>
+      <c r="O25" s="11"/>
+      <c r="P25" s="12" t="s">
         <v>38</v>
       </c>
-      <c r="Q25" s="5" t="s">
+      <c r="Q25" s="21" t="s">
         <v>344</v>
+      </c>
+      <c r="R25" s="15"/>
+      <c r="S25" s="16" t="s">
+        <v>365</v>
       </c>
     </row>
     <row r="26" spans="1:19" ht="45" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
changed 0154005.DR Littlefuse_154_Fuse (F1) to 30775 out of TE.DbLib/FUSE, 744235900 (L5) to 30776 out of TE.DbLib/L_SMD
</commit_message>
<xml_diff>
--- a/Using Trenz Library/BOM_MissingComponents_in_process_Simon.xlsx
+++ b/Using Trenz Library/BOM_MissingComponents_in_process_Simon.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="647" uniqueCount="366">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="648" uniqueCount="367">
   <si>
     <t>Quantity</t>
   </si>
@@ -1125,6 +1125,9 @@
   </si>
   <si>
     <t>used NLV74HC32ADTR2G</t>
+  </si>
+  <si>
+    <t>used 744235900</t>
   </si>
 </sst>
 </file>
@@ -2163,103 +2166,109 @@
       <c r="S10" s="14"/>
     </row>
     <row r="11" spans="1:19" ht="45" x14ac:dyDescent="0.25">
-      <c r="A11" s="3">
+      <c r="A11" s="11">
         <v>1</v>
       </c>
-      <c r="B11" s="4" t="s">
+      <c r="B11" s="12" t="s">
         <v>16</v>
       </c>
-      <c r="C11" s="4" t="s">
+      <c r="C11" s="12" t="s">
         <v>17</v>
       </c>
-      <c r="D11" s="4" t="s">
+      <c r="D11" s="12" t="s">
         <v>18</v>
       </c>
-      <c r="E11" s="4" t="s">
+      <c r="E11" s="12" t="s">
         <v>19</v>
       </c>
-      <c r="F11" s="4" t="s">
+      <c r="F11" s="12" t="s">
         <v>16</v>
       </c>
-      <c r="G11" s="4" t="s">
+      <c r="G11" s="12" t="s">
         <v>20</v>
       </c>
-      <c r="H11" s="4" t="s">
+      <c r="H11" s="12" t="s">
         <v>21</v>
       </c>
-      <c r="I11" s="4" t="s">
+      <c r="I11" s="12" t="s">
         <v>22</v>
       </c>
-      <c r="J11" s="4" t="s">
+      <c r="J11" s="12" t="s">
         <v>23</v>
       </c>
-      <c r="K11" s="4" t="s">
+      <c r="K11" s="12" t="s">
         <v>24</v>
       </c>
-      <c r="L11" s="4" t="s">
+      <c r="L11" s="12" t="s">
         <v>25</v>
       </c>
-      <c r="M11" s="4" t="s">
+      <c r="M11" s="12" t="s">
         <v>26</v>
       </c>
-      <c r="N11" s="3"/>
-      <c r="O11" s="3"/>
-      <c r="P11" s="4" t="s">
+      <c r="N11" s="11"/>
+      <c r="O11" s="11"/>
+      <c r="P11" s="12" t="s">
         <v>27</v>
       </c>
-      <c r="Q11" s="5" t="s">
+      <c r="Q11" s="21" t="s">
         <v>323</v>
       </c>
+      <c r="R11" s="15"/>
+      <c r="S11" s="14"/>
     </row>
     <row r="12" spans="1:19" ht="45" x14ac:dyDescent="0.25">
-      <c r="A12" s="3">
+      <c r="A12" s="11">
         <v>2</v>
       </c>
-      <c r="B12" s="4" t="s">
+      <c r="B12" s="12" t="s">
         <v>162</v>
       </c>
-      <c r="C12" s="4" t="s">
+      <c r="C12" s="12" t="s">
         <v>163</v>
       </c>
-      <c r="D12" s="4" t="s">
+      <c r="D12" s="12" t="s">
         <v>58</v>
       </c>
-      <c r="E12" s="4" t="s">
+      <c r="E12" s="12" t="s">
         <v>162</v>
       </c>
-      <c r="F12" s="4" t="s">
+      <c r="F12" s="12" t="s">
         <v>162</v>
       </c>
-      <c r="G12" s="4" t="s">
+      <c r="G12" s="12" t="s">
         <v>164</v>
       </c>
-      <c r="H12" s="4" t="s">
+      <c r="H12" s="12" t="s">
         <v>165</v>
       </c>
-      <c r="I12" s="3"/>
-      <c r="J12" s="4" t="s">
+      <c r="I12" s="11"/>
+      <c r="J12" s="12" t="s">
         <v>23</v>
       </c>
-      <c r="K12" s="4" t="s">
+      <c r="K12" s="12" t="s">
         <v>166</v>
       </c>
-      <c r="L12" s="4" t="s">
+      <c r="L12" s="12" t="s">
         <v>25</v>
       </c>
-      <c r="M12" s="4" t="s">
+      <c r="M12" s="12" t="s">
         <v>167</v>
       </c>
-      <c r="N12" s="4" t="s">
+      <c r="N12" s="12" t="s">
         <v>36</v>
       </c>
-      <c r="O12" s="4" t="s">
+      <c r="O12" s="12" t="s">
         <v>168</v>
       </c>
-      <c r="P12" s="4" t="s">
-        <v>47</v>
-      </c>
-      <c r="Q12" s="5" t="s">
+      <c r="P12" s="12" t="s">
+        <v>47</v>
+      </c>
+      <c r="Q12" s="21" t="s">
         <v>331</v>
+      </c>
+      <c r="R12" s="15"/>
+      <c r="S12" s="23" t="s">
+        <v>366</v>
       </c>
     </row>
     <row r="13" spans="1:19" ht="45" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
changed 4k99 R_0603 resistors (R50,R56) to 22754 out of TE.DbLib/R_1005_0402, 150060BS75000 (D12,D24) to 30779 out of TE.DbLib/LED
</commit_message>
<xml_diff>
--- a/Using Trenz Library/BOM_MissingComponents_in_process_Simon.xlsx
+++ b/Using Trenz Library/BOM_MissingComponents_in_process_Simon.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="648" uniqueCount="367">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="651" uniqueCount="369">
   <si>
     <t>Quantity</t>
   </si>
@@ -1128,13 +1128,19 @@
   </si>
   <si>
     <t>used 744235900</t>
+  </si>
+  <si>
+    <t>used 150060BS75000</t>
+  </si>
+  <si>
+    <t xml:space="preserve">used 3x100uF </t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1160,6 +1166,12 @@
     <font>
       <sz val="11"/>
       <color theme="9"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -1265,7 +1277,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="27">
+  <cellXfs count="30">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1316,7 +1328,6 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
@@ -1328,6 +1339,16 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" quotePrefix="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1691,53 +1712,56 @@
       <c r="R1" s="6"/>
     </row>
     <row r="2" spans="1:19" ht="45" x14ac:dyDescent="0.25">
-      <c r="A2" s="3">
+      <c r="A2" s="26">
         <v>3</v>
       </c>
-      <c r="B2" s="4" t="s">
+      <c r="B2" s="27" t="s">
         <v>210</v>
       </c>
-      <c r="C2" s="4" t="s">
+      <c r="C2" s="27" t="s">
         <v>211</v>
       </c>
-      <c r="D2" s="4" t="s">
+      <c r="D2" s="27" t="s">
         <v>58</v>
       </c>
-      <c r="E2" s="4" t="s">
+      <c r="E2" s="27" t="s">
         <v>212</v>
       </c>
-      <c r="F2" s="4" t="s">
+      <c r="F2" s="27" t="s">
         <v>210</v>
       </c>
-      <c r="G2" s="4" t="s">
+      <c r="G2" s="27" t="s">
         <v>213</v>
       </c>
-      <c r="H2" s="4" t="s">
+      <c r="H2" s="27" t="s">
         <v>214</v>
       </c>
-      <c r="I2" s="3"/>
-      <c r="J2" s="4" t="s">
+      <c r="I2" s="26"/>
+      <c r="J2" s="27" t="s">
         <v>23</v>
       </c>
-      <c r="K2" s="4" t="s">
+      <c r="K2" s="27" t="s">
         <v>215</v>
       </c>
-      <c r="L2" s="4" t="s">
+      <c r="L2" s="27" t="s">
         <v>25</v>
       </c>
-      <c r="M2" s="4" t="s">
+      <c r="M2" s="27" t="s">
         <v>216</v>
       </c>
-      <c r="N2" s="3"/>
-      <c r="O2" s="3"/>
-      <c r="P2" s="4" t="s">
-        <v>47</v>
-      </c>
-      <c r="Q2" s="22" t="s">
+      <c r="N2" s="26"/>
+      <c r="O2" s="26"/>
+      <c r="P2" s="27" t="s">
+        <v>47</v>
+      </c>
+      <c r="Q2" s="28" t="s">
         <v>320</v>
       </c>
-      <c r="R2" s="7" t="s">
+      <c r="R2" s="29" t="s">
         <v>326</v>
+      </c>
+      <c r="S2" s="19" t="s">
+        <v>368</v>
       </c>
     </row>
     <row r="3" spans="1:19" ht="45" x14ac:dyDescent="0.25">
@@ -1851,56 +1875,60 @@
       <c r="S4" s="14"/>
     </row>
     <row r="5" spans="1:19" ht="45" x14ac:dyDescent="0.25">
-      <c r="A5" s="3">
+      <c r="A5" s="11">
         <v>5</v>
       </c>
-      <c r="B5" s="4" t="s">
+      <c r="B5" s="12" t="s">
         <v>256</v>
       </c>
-      <c r="C5" s="4" t="s">
+      <c r="C5" s="12" t="s">
         <v>257</v>
       </c>
-      <c r="D5" s="4" t="s">
+      <c r="D5" s="12" t="s">
         <v>58</v>
       </c>
-      <c r="E5" s="4" t="s">
+      <c r="E5" s="12" t="s">
         <v>256</v>
       </c>
-      <c r="F5" s="4" t="s">
+      <c r="F5" s="12" t="s">
         <v>256</v>
       </c>
-      <c r="G5" s="4" t="s">
+      <c r="G5" s="12" t="s">
         <v>258</v>
       </c>
-      <c r="H5" s="4" t="s">
+      <c r="H5" s="12" t="s">
         <v>158</v>
       </c>
-      <c r="I5" s="4" t="s">
+      <c r="I5" s="12" t="s">
         <v>54</v>
       </c>
-      <c r="J5" s="4" t="s">
+      <c r="J5" s="12" t="s">
         <v>23</v>
       </c>
-      <c r="K5" s="4" t="s">
+      <c r="K5" s="12" t="s">
         <v>259</v>
       </c>
-      <c r="L5" s="4" t="s">
+      <c r="L5" s="12" t="s">
         <v>25</v>
       </c>
-      <c r="M5" s="4" t="s">
+      <c r="M5" s="12" t="s">
         <v>260</v>
       </c>
-      <c r="N5" s="4" t="s">
+      <c r="N5" s="12" t="s">
         <v>36</v>
       </c>
-      <c r="O5" s="4" t="s">
+      <c r="O5" s="12" t="s">
         <v>261</v>
       </c>
-      <c r="P5" s="4" t="s">
-        <v>47</v>
-      </c>
-      <c r="Q5" s="5" t="s">
+      <c r="P5" s="12" t="s">
+        <v>47</v>
+      </c>
+      <c r="Q5" s="21" t="s">
         <v>327</v>
+      </c>
+      <c r="R5" s="15"/>
+      <c r="S5" s="22" t="s">
+        <v>367</v>
       </c>
     </row>
     <row r="6" spans="1:19" ht="60" x14ac:dyDescent="0.25">
@@ -2267,7 +2295,7 @@
         <v>331</v>
       </c>
       <c r="R12" s="15"/>
-      <c r="S12" s="23" t="s">
+      <c r="S12" s="22" t="s">
         <v>366</v>
       </c>
     </row>
@@ -2409,51 +2437,54 @@
       </c>
     </row>
     <row r="16" spans="1:19" ht="45" x14ac:dyDescent="0.25">
-      <c r="A16" s="3">
+      <c r="A16" s="11">
         <v>2</v>
       </c>
-      <c r="B16" s="4" t="s">
+      <c r="B16" s="12" t="s">
         <v>151</v>
       </c>
-      <c r="C16" s="4" t="s">
+      <c r="C16" s="12" t="s">
         <v>152</v>
       </c>
-      <c r="D16" s="4" t="s">
+      <c r="D16" s="12" t="s">
         <v>41</v>
       </c>
-      <c r="E16" s="4" t="s">
+      <c r="E16" s="12" t="s">
         <v>153</v>
       </c>
-      <c r="F16" s="4" t="s">
+      <c r="F16" s="12" t="s">
         <v>151</v>
       </c>
-      <c r="G16" s="4" t="s">
+      <c r="G16" s="12" t="s">
         <v>52</v>
       </c>
-      <c r="H16" s="4" t="s">
+      <c r="H16" s="12" t="s">
         <v>53</v>
       </c>
-      <c r="I16" s="4" t="s">
+      <c r="I16" s="12" t="s">
         <v>54</v>
       </c>
-      <c r="J16" s="4" t="s">
+      <c r="J16" s="12" t="s">
         <v>23</v>
       </c>
-      <c r="K16" s="4" t="s">
+      <c r="K16" s="12" t="s">
         <v>154</v>
       </c>
-      <c r="L16" s="3"/>
-      <c r="M16" s="3"/>
-      <c r="N16" s="3"/>
-      <c r="O16" s="3"/>
-      <c r="P16" s="4" t="s">
-        <v>47</v>
-      </c>
-      <c r="Q16" t="s">
+      <c r="L16" s="11"/>
+      <c r="M16" s="11"/>
+      <c r="N16" s="11"/>
+      <c r="O16" s="11"/>
+      <c r="P16" s="12" t="s">
+        <v>47</v>
+      </c>
+      <c r="Q16" s="14" t="s">
         <v>324</v>
       </c>
-      <c r="R16" s="7" t="s">
+      <c r="R16" s="15" t="s">
         <v>335</v>
+      </c>
+      <c r="S16" s="19" t="s">
+        <v>355</v>
       </c>
     </row>
     <row r="17" spans="1:19" ht="210" x14ac:dyDescent="0.25">
@@ -2958,7 +2989,7 @@
       <c r="R26" s="15" t="s">
         <v>348</v>
       </c>
-      <c r="S26" s="23" t="s">
+      <c r="S26" s="22" t="s">
         <v>363</v>
       </c>
     </row>
@@ -3128,7 +3159,7 @@
       <c r="A30" s="3">
         <v>5</v>
       </c>
-      <c r="B30" s="26" t="s">
+      <c r="B30" s="25" t="s">
         <v>268</v>
       </c>
       <c r="C30" s="4" t="s">
@@ -3278,7 +3309,7 @@
       <c r="P32" s="12" t="s">
         <v>47</v>
       </c>
-      <c r="Q32" s="25" t="s">
+      <c r="Q32" s="24" t="s">
         <v>334</v>
       </c>
       <c r="R32" s="15"/>
@@ -3327,7 +3358,7 @@
       <c r="P33" s="12" t="s">
         <v>47</v>
       </c>
-      <c r="Q33" s="25" t="s">
+      <c r="Q33" s="24" t="s">
         <v>334</v>
       </c>
       <c r="R33" s="15"/>
@@ -3374,7 +3405,7 @@
       <c r="P34" s="12" t="s">
         <v>47</v>
       </c>
-      <c r="Q34" s="25" t="s">
+      <c r="Q34" s="24" t="s">
         <v>334</v>
       </c>
       <c r="R34" s="15"/>
@@ -3480,7 +3511,7 @@
         <v>323</v>
       </c>
       <c r="R36" s="15"/>
-      <c r="S36" s="23" t="s">
+      <c r="S36" s="22" t="s">
         <v>360</v>
       </c>
     </row>
@@ -3535,7 +3566,7 @@
         <v>323</v>
       </c>
       <c r="R37" s="15"/>
-      <c r="S37" s="23" t="s">
+      <c r="S37" s="22" t="s">
         <v>360</v>
       </c>
     </row>
@@ -3590,7 +3621,7 @@
         <v>323</v>
       </c>
       <c r="R38" s="15"/>
-      <c r="S38" s="23" t="s">
+      <c r="S38" s="22" t="s">
         <v>360</v>
       </c>
     </row>
@@ -3645,7 +3676,7 @@
         <v>323</v>
       </c>
       <c r="R39" s="15"/>
-      <c r="S39" s="23" t="s">
+      <c r="S39" s="22" t="s">
         <v>360</v>
       </c>
     </row>
@@ -3808,7 +3839,7 @@
         <v>323</v>
       </c>
       <c r="R42" s="15"/>
-      <c r="S42" s="24" t="s">
+      <c r="S42" s="23" t="s">
         <v>361</v>
       </c>
     </row>
@@ -3863,7 +3894,7 @@
         <v>323</v>
       </c>
       <c r="R43" s="15"/>
-      <c r="S43" s="24" t="s">
+      <c r="S43" s="23" t="s">
         <v>362</v>
       </c>
     </row>

</xml_diff>

<commit_message>
changed LA4128V-75TN100E (U4) to 30780 out of TE.DbLib/PROG_LOGIC
</commit_message>
<xml_diff>
--- a/Using Trenz Library/BOM_MissingComponents_in_process_Simon.xlsx
+++ b/Using Trenz Library/BOM_MissingComponents_in_process_Simon.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="651" uniqueCount="369">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="652" uniqueCount="370">
   <si>
     <t>Quantity</t>
   </si>
@@ -1134,6 +1134,9 @@
   </si>
   <si>
     <t xml:space="preserve">used 3x100uF </t>
+  </si>
+  <si>
+    <t>used TPS54260QDGQRQ1</t>
   </si>
 </sst>
 </file>
@@ -1177,7 +1180,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1193,12 +1196,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FF92D050"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFF0000"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1277,7 +1274,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="30">
+  <cellXfs count="29">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1335,9 +1332,6 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" quotePrefix="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1712,52 +1706,52 @@
       <c r="R1" s="6"/>
     </row>
     <row r="2" spans="1:19" ht="45" x14ac:dyDescent="0.25">
-      <c r="A2" s="26">
+      <c r="A2" s="25">
         <v>3</v>
       </c>
-      <c r="B2" s="27" t="s">
+      <c r="B2" s="26" t="s">
         <v>210</v>
       </c>
-      <c r="C2" s="27" t="s">
+      <c r="C2" s="26" t="s">
         <v>211</v>
       </c>
-      <c r="D2" s="27" t="s">
+      <c r="D2" s="26" t="s">
         <v>58</v>
       </c>
-      <c r="E2" s="27" t="s">
+      <c r="E2" s="26" t="s">
         <v>212</v>
       </c>
-      <c r="F2" s="27" t="s">
+      <c r="F2" s="26" t="s">
         <v>210</v>
       </c>
-      <c r="G2" s="27" t="s">
+      <c r="G2" s="26" t="s">
         <v>213</v>
       </c>
-      <c r="H2" s="27" t="s">
+      <c r="H2" s="26" t="s">
         <v>214</v>
       </c>
-      <c r="I2" s="26"/>
-      <c r="J2" s="27" t="s">
+      <c r="I2" s="25"/>
+      <c r="J2" s="26" t="s">
         <v>23</v>
       </c>
-      <c r="K2" s="27" t="s">
+      <c r="K2" s="26" t="s">
         <v>215</v>
       </c>
-      <c r="L2" s="27" t="s">
+      <c r="L2" s="26" t="s">
         <v>25</v>
       </c>
-      <c r="M2" s="27" t="s">
+      <c r="M2" s="26" t="s">
         <v>216</v>
       </c>
-      <c r="N2" s="26"/>
-      <c r="O2" s="26"/>
-      <c r="P2" s="27" t="s">
-        <v>47</v>
-      </c>
-      <c r="Q2" s="28" t="s">
+      <c r="N2" s="25"/>
+      <c r="O2" s="25"/>
+      <c r="P2" s="26" t="s">
+        <v>47</v>
+      </c>
+      <c r="Q2" s="27" t="s">
         <v>320</v>
       </c>
-      <c r="R2" s="29" t="s">
+      <c r="R2" s="28" t="s">
         <v>326</v>
       </c>
       <c r="S2" s="19" t="s">
@@ -2994,59 +2988,62 @@
       </c>
     </row>
     <row r="27" spans="1:19" ht="90" x14ac:dyDescent="0.25">
-      <c r="A27" s="3">
+      <c r="A27" s="11">
         <v>1</v>
       </c>
-      <c r="B27" s="4" t="s">
+      <c r="B27" s="12" t="s">
         <v>142</v>
       </c>
-      <c r="C27" s="4" t="s">
+      <c r="C27" s="12" t="s">
         <v>143</v>
       </c>
-      <c r="D27" s="4" t="s">
+      <c r="D27" s="12" t="s">
         <v>118</v>
       </c>
-      <c r="E27" s="4" t="s">
+      <c r="E27" s="12" t="s">
         <v>144</v>
       </c>
-      <c r="F27" s="4" t="s">
+      <c r="F27" s="12" t="s">
         <v>142</v>
       </c>
-      <c r="G27" s="4" t="s">
+      <c r="G27" s="12" t="s">
         <v>145</v>
       </c>
-      <c r="H27" s="4" t="s">
+      <c r="H27" s="12" t="s">
         <v>146</v>
       </c>
-      <c r="I27" s="4" t="s">
+      <c r="I27" s="12" t="s">
         <v>147</v>
       </c>
-      <c r="J27" s="4" t="s">
+      <c r="J27" s="12" t="s">
         <v>23</v>
       </c>
-      <c r="K27" s="4" t="s">
+      <c r="K27" s="12" t="s">
         <v>148</v>
       </c>
-      <c r="L27" s="4" t="s">
+      <c r="L27" s="12" t="s">
         <v>25</v>
       </c>
-      <c r="M27" s="4" t="s">
+      <c r="M27" s="12" t="s">
         <v>149</v>
       </c>
-      <c r="N27" s="4" t="s">
+      <c r="N27" s="12" t="s">
         <v>36</v>
       </c>
-      <c r="O27" s="4" t="s">
+      <c r="O27" s="12" t="s">
         <v>150</v>
       </c>
-      <c r="P27" s="4" t="s">
-        <v>47</v>
-      </c>
-      <c r="Q27" s="5" t="s">
+      <c r="P27" s="12" t="s">
+        <v>47</v>
+      </c>
+      <c r="Q27" s="21" t="s">
         <v>346</v>
       </c>
-      <c r="R27" s="7" t="s">
+      <c r="R27" s="15" t="s">
         <v>345</v>
+      </c>
+      <c r="S27" s="22" t="s">
+        <v>369</v>
       </c>
     </row>
     <row r="28" spans="1:19" ht="45" x14ac:dyDescent="0.25">
@@ -3156,53 +3153,55 @@
       <c r="S29" s="14"/>
     </row>
     <row r="30" spans="1:19" ht="45" x14ac:dyDescent="0.25">
-      <c r="A30" s="3">
+      <c r="A30" s="11">
         <v>5</v>
       </c>
-      <c r="B30" s="25" t="s">
+      <c r="B30" s="12" t="s">
         <v>268</v>
       </c>
-      <c r="C30" s="4" t="s">
+      <c r="C30" s="12" t="s">
         <v>269</v>
       </c>
-      <c r="D30" s="4" t="s">
+      <c r="D30" s="12" t="s">
         <v>270</v>
       </c>
-      <c r="E30" s="4" t="s">
+      <c r="E30" s="12" t="s">
         <v>268</v>
       </c>
-      <c r="F30" s="4" t="s">
+      <c r="F30" s="12" t="s">
         <v>268</v>
       </c>
-      <c r="G30" s="4" t="s">
+      <c r="G30" s="12" t="s">
         <v>271</v>
       </c>
-      <c r="H30" s="4" t="s">
+      <c r="H30" s="12" t="s">
         <v>272</v>
       </c>
-      <c r="I30" s="4" t="s">
+      <c r="I30" s="12" t="s">
         <v>273</v>
       </c>
-      <c r="J30" s="4" t="s">
+      <c r="J30" s="12" t="s">
         <v>25</v>
       </c>
-      <c r="K30" s="4" t="s">
+      <c r="K30" s="12" t="s">
         <v>274</v>
       </c>
-      <c r="L30" s="4" t="s">
+      <c r="L30" s="12" t="s">
         <v>36</v>
       </c>
-      <c r="M30" s="4" t="s">
+      <c r="M30" s="12" t="s">
         <v>275</v>
       </c>
-      <c r="N30" s="3"/>
-      <c r="O30" s="3"/>
-      <c r="P30" s="4" t="s">
-        <v>47</v>
-      </c>
-      <c r="Q30" s="5" t="s">
+      <c r="N30" s="11"/>
+      <c r="O30" s="11"/>
+      <c r="P30" s="12" t="s">
+        <v>47</v>
+      </c>
+      <c r="Q30" s="21" t="s">
         <v>323</v>
       </c>
+      <c r="R30" s="15"/>
+      <c r="S30" s="14"/>
     </row>
     <row r="31" spans="1:19" ht="60" x14ac:dyDescent="0.25">
       <c r="A31" s="11">

</xml_diff>

<commit_message>
- changed TXS0108EQPWRQ1 (U14,U25,U30) to 30791 out of TE.DbLib/A_IF - removed R149, R225, R211 (level shifter)
</commit_message>
<xml_diff>
--- a/Using Trenz Library/BOM_MissingComponents_in_process_Simon.xlsx
+++ b/Using Trenz Library/BOM_MissingComponents_in_process_Simon.xlsx
@@ -2831,53 +2831,55 @@
       </c>
     </row>
     <row r="24" spans="1:19" ht="45" x14ac:dyDescent="0.25">
-      <c r="A24" s="3">
+      <c r="A24" s="11">
         <v>3</v>
       </c>
-      <c r="B24" s="4" t="s">
+      <c r="B24" s="12" t="s">
         <v>224</v>
       </c>
-      <c r="C24" s="4" t="s">
+      <c r="C24" s="12" t="s">
         <v>225</v>
       </c>
-      <c r="D24" s="4" t="s">
+      <c r="D24" s="12" t="s">
         <v>118</v>
       </c>
-      <c r="E24" s="4" t="s">
+      <c r="E24" s="12" t="s">
         <v>224</v>
       </c>
-      <c r="F24" s="4" t="s">
+      <c r="F24" s="12" t="s">
         <v>224</v>
       </c>
-      <c r="G24" s="4" t="s">
+      <c r="G24" s="12" t="s">
         <v>226</v>
       </c>
-      <c r="H24" s="4" t="s">
+      <c r="H24" s="12" t="s">
         <v>227</v>
       </c>
-      <c r="I24" s="4" t="s">
+      <c r="I24" s="12" t="s">
         <v>228</v>
       </c>
-      <c r="J24" s="4" t="s">
+      <c r="J24" s="12" t="s">
         <v>25</v>
       </c>
-      <c r="K24" s="4" t="s">
+      <c r="K24" s="12" t="s">
         <v>229</v>
       </c>
-      <c r="L24" s="4" t="s">
+      <c r="L24" s="12" t="s">
         <v>36</v>
       </c>
-      <c r="M24" s="4" t="s">
+      <c r="M24" s="12" t="s">
         <v>230</v>
       </c>
-      <c r="N24" s="3"/>
-      <c r="O24" s="3"/>
-      <c r="P24" s="4" t="s">
-        <v>47</v>
-      </c>
-      <c r="Q24" t="s">
+      <c r="N24" s="11"/>
+      <c r="O24" s="11"/>
+      <c r="P24" s="12" t="s">
+        <v>47</v>
+      </c>
+      <c r="Q24" s="14" t="s">
         <v>334</v>
       </c>
+      <c r="R24" s="15"/>
+      <c r="S24" s="14"/>
     </row>
     <row r="25" spans="1:19" ht="60" x14ac:dyDescent="0.25">
       <c r="A25" s="11">

</xml_diff>

<commit_message>
- changed BZX84C15 (D22) to 29229 (MMSZ5242BT1G) out of TE.DbLib/DIODE - changed C121 10uF 35V to 10uF 50V (1206) - changed C72 47uF 16V to 47uF 6.3V (0805) - changed C1 22uF 25V to 100uF 6.3V (1206)
</commit_message>
<xml_diff>
--- a/Using Trenz Library/BOM_MissingComponents_in_process_Simon.xlsx
+++ b/Using Trenz Library/BOM_MissingComponents_in_process_Simon.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="652" uniqueCount="370">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="653" uniqueCount="371">
   <si>
     <t>Quantity</t>
   </si>
@@ -1137,6 +1137,9 @@
   </si>
   <si>
     <t>used TPS54260QDGQRQ1</t>
+  </si>
+  <si>
+    <t>used MMSZ5242BT1G</t>
   </si>
 </sst>
 </file>
@@ -1200,7 +1203,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="6">
+  <borders count="7">
     <border>
       <left/>
       <right/>
@@ -1269,12 +1272,27 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFFF0000"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFFF0000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFFF0000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFFF0000"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="29">
+  <cellXfs count="30">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1343,6 +1361,9 @@
     <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1985,56 +2006,60 @@
       </c>
     </row>
     <row r="7" spans="1:19" ht="45" x14ac:dyDescent="0.25">
-      <c r="A7" s="3">
+      <c r="A7" s="11">
         <v>1</v>
       </c>
-      <c r="B7" s="4" t="s">
+      <c r="B7" s="12" t="s">
         <v>74</v>
       </c>
-      <c r="C7" s="4" t="s">
+      <c r="C7" s="12" t="s">
         <v>75</v>
       </c>
-      <c r="D7" s="4" t="s">
+      <c r="D7" s="12" t="s">
         <v>76</v>
       </c>
-      <c r="E7" s="4" t="s">
+      <c r="E7" s="12" t="s">
         <v>77</v>
       </c>
-      <c r="F7" s="4" t="s">
+      <c r="F7" s="12" t="s">
         <v>74</v>
       </c>
-      <c r="G7" s="4" t="s">
+      <c r="G7" s="12" t="s">
         <v>78</v>
       </c>
-      <c r="H7" s="4" t="s">
+      <c r="H7" s="12" t="s">
         <v>79</v>
       </c>
-      <c r="I7" s="4" t="s">
+      <c r="I7" s="12" t="s">
         <v>80</v>
       </c>
-      <c r="J7" s="4" t="s">
+      <c r="J7" s="12" t="s">
         <v>25</v>
       </c>
-      <c r="K7" s="4" t="s">
+      <c r="K7" s="12" t="s">
         <v>81</v>
       </c>
-      <c r="L7" s="4" t="s">
+      <c r="L7" s="12" t="s">
         <v>36</v>
       </c>
-      <c r="M7" s="4" t="s">
+      <c r="M7" s="12" t="s">
         <v>82</v>
       </c>
-      <c r="N7" s="4" t="s">
+      <c r="N7" s="12" t="s">
         <v>23</v>
       </c>
-      <c r="O7" s="4" t="s">
+      <c r="O7" s="12" t="s">
         <v>83</v>
       </c>
-      <c r="P7" s="4" t="s">
-        <v>47</v>
-      </c>
-      <c r="Q7" t="s">
+      <c r="P7" s="12" t="s">
+        <v>47</v>
+      </c>
+      <c r="Q7" s="14" t="s">
         <v>349</v>
+      </c>
+      <c r="R7" s="15"/>
+      <c r="S7" s="29" t="s">
+        <v>370</v>
       </c>
     </row>
     <row r="8" spans="1:19" ht="30" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
- changed R127, R164 to 26473 (6k98 R_0603) out of TE.DbLib/R_1608_0603 and R126, R161 to 22655 (12k R_0603) out of TE.DbLib/R_1608_0603 to get ratio of 1.7 (3V3) - changed R81 to 26473 (6k98 R_0603) out of TE.DbLib/R_1608_0603 and R80 to 26540 (22k R_0603) out of TE.DbLib/R_1608_0603 to get ratio of 3.1 (5V)
</commit_message>
<xml_diff>
--- a/Using Trenz Library/BOM_MissingComponents_in_process_Simon.xlsx
+++ b/Using Trenz Library/BOM_MissingComponents_in_process_Simon.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="653" uniqueCount="371">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="654" uniqueCount="372">
   <si>
     <t>Quantity</t>
   </si>
@@ -1140,6 +1140,9 @@
   </si>
   <si>
     <t>used MMSZ5242BT1G</t>
+  </si>
+  <si>
+    <t>see commit -&gt; ratios should be even better</t>
   </si>
 </sst>
 </file>
@@ -2604,49 +2607,53 @@
       <c r="R18" s="15"/>
       <c r="S18" s="14"/>
     </row>
-    <row r="19" spans="1:19" ht="30" x14ac:dyDescent="0.25">
-      <c r="A19" s="3">
+    <row r="19" spans="1:19" ht="45" x14ac:dyDescent="0.25">
+      <c r="A19" s="11">
         <v>4</v>
       </c>
-      <c r="B19" s="4" t="s">
+      <c r="B19" s="12" t="s">
         <v>231</v>
       </c>
-      <c r="C19" s="4" t="s">
+      <c r="C19" s="12" t="s">
         <v>232</v>
       </c>
-      <c r="D19" s="4" t="s">
+      <c r="D19" s="12" t="s">
         <v>50</v>
       </c>
-      <c r="E19" s="4" t="s">
+      <c r="E19" s="12" t="s">
         <v>233</v>
       </c>
-      <c r="F19" s="4" t="s">
+      <c r="F19" s="12" t="s">
         <v>231</v>
       </c>
-      <c r="G19" s="4" t="s">
+      <c r="G19" s="12" t="s">
         <v>52</v>
       </c>
-      <c r="H19" s="4" t="s">
+      <c r="H19" s="12" t="s">
         <v>53</v>
       </c>
-      <c r="I19" s="4" t="s">
+      <c r="I19" s="12" t="s">
         <v>54</v>
       </c>
-      <c r="J19" s="4" t="s">
+      <c r="J19" s="12" t="s">
         <v>23</v>
       </c>
-      <c r="K19" s="4" t="s">
+      <c r="K19" s="12" t="s">
         <v>234</v>
       </c>
-      <c r="L19" s="3"/>
-      <c r="M19" s="3"/>
-      <c r="N19" s="3"/>
-      <c r="O19" s="3"/>
-      <c r="P19" s="4" t="s">
-        <v>47</v>
-      </c>
-      <c r="Q19" t="s">
+      <c r="L19" s="11"/>
+      <c r="M19" s="11"/>
+      <c r="N19" s="11"/>
+      <c r="O19" s="11"/>
+      <c r="P19" s="12" t="s">
+        <v>47</v>
+      </c>
+      <c r="Q19" s="14" t="s">
         <v>335</v>
+      </c>
+      <c r="R19" s="15"/>
+      <c r="S19" s="16" t="s">
+        <v>371</v>
       </c>
     </row>
     <row r="20" spans="1:19" ht="45" x14ac:dyDescent="0.25">

</xml_diff>